<commit_message>
SD card and 3.3uH IND updated in lob, schematic and PCB. BOM also updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SaleemD-CustomProduct\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{336B9EA2-4AD8-4869-98A0-34BA03B50A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,17 +18,24 @@
   <definedNames>
     <definedName name="LCSC">Sheet1!$N$20</definedName>
   </definedNames>
-  <calcPr calcId="162913" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="244">
   <si>
     <t>S. No.</t>
   </si>
@@ -222,9 +230,6 @@
   </si>
   <si>
     <t>06035A100JAT2A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KYOCERA </t>
   </si>
   <si>
     <t>CAP CER 20PF 50V C0G/NP0 0603</t>
@@ -270,13 +275,7 @@
     <t xml:space="preserve">Vishay </t>
   </si>
   <si>
-    <t>FIXED IND 3.3UH 6.5A 36 MOHM SMD</t>
-  </si>
-  <si>
     <t>L1</t>
-  </si>
-  <si>
-    <t>ASPI-0530LR-3R3M-T2</t>
   </si>
   <si>
     <t xml:space="preserve">Abracon </t>
@@ -539,9 +538,6 @@
     <t>J6</t>
   </si>
   <si>
-    <t>114-00841-68</t>
-  </si>
-  <si>
     <t xml:space="preserve">Amphenol </t>
   </si>
   <si>
@@ -656,9 +652,6 @@
     <t>C76615</t>
   </si>
   <si>
-    <t>Utsource</t>
-  </si>
-  <si>
     <t>C1648</t>
   </si>
   <si>
@@ -744,17 +737,53 @@
   </si>
   <si>
     <t>C132563</t>
+  </si>
+  <si>
+    <t>AVX</t>
+  </si>
+  <si>
+    <t>CC0603JRNPO9BN100</t>
+  </si>
+  <si>
+    <t>BZT52C3V3S</t>
+  </si>
+  <si>
+    <t>C231329</t>
+  </si>
+  <si>
+    <t>C173439</t>
+  </si>
+  <si>
+    <t>C106245</t>
+  </si>
+  <si>
+    <t>Awaiting reponse of custom supplier</t>
+  </si>
+  <si>
+    <t>C125616</t>
+  </si>
+  <si>
+    <t>TF-002T-15</t>
+  </si>
+  <si>
+    <t>FIXED IND 3.3UH 6A 36 MOHM SMD</t>
+  </si>
+  <si>
+    <t>IHLP2525CZER3R3M01</t>
+  </si>
+  <si>
+    <t>C506574</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00000"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00000"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1240,7 +1269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1390,168 +1419,204 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="21" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1833,7 +1898,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1859,28 +1924,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="102" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="105"/>
-      <c r="C1" s="105"/>
-      <c r="D1" s="105"/>
-      <c r="E1" s="105"/>
-      <c r="F1" s="105"/>
-      <c r="G1" s="105"/>
-      <c r="H1" s="105"/>
-      <c r="I1" s="105"/>
-      <c r="J1" s="105"/>
-      <c r="K1" s="105"/>
-      <c r="L1" s="105"/>
-      <c r="M1" s="105"/>
-      <c r="N1" s="105"/>
-      <c r="O1" s="105"/>
-      <c r="P1" s="105"/>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105"/>
-      <c r="T1" s="106"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="103"/>
+      <c r="L1" s="103"/>
+      <c r="M1" s="103"/>
+      <c r="N1" s="103"/>
+      <c r="O1" s="103"/>
+      <c r="P1" s="103"/>
+      <c r="Q1" s="103"/>
+      <c r="R1" s="103"/>
+      <c r="S1" s="103"/>
+      <c r="T1" s="104"/>
     </row>
     <row r="2" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
@@ -1948,7 +2013,7 @@
       <c r="A3" s="33">
         <v>1</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="98" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -1967,46 +2032,46 @@
         <v>34</v>
       </c>
       <c r="H3" s="50" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="I3" s="47" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="K3" s="58">
+        <v>169</v>
+      </c>
+      <c r="K3" s="53">
         <v>10</v>
       </c>
-      <c r="L3" s="73">
+      <c r="L3" s="68">
         <v>1</v>
       </c>
-      <c r="M3" s="58">
+      <c r="M3" s="53">
         <f>L3*5</f>
         <v>5</v>
       </c>
-      <c r="N3" s="59" t="s">
-        <v>196</v>
-      </c>
-      <c r="O3" s="60">
+      <c r="N3" s="54" t="s">
+        <v>192</v>
+      </c>
+      <c r="O3" s="55">
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="P3" s="61">
+      <c r="P3" s="56">
         <f>O3*L3</f>
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="Q3" s="61">
+      <c r="Q3" s="56">
         <f>O3*K3</f>
         <v>0.60899999999999999</v>
       </c>
-      <c r="R3" s="60">
+      <c r="R3" s="55">
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="S3" s="61">
+      <c r="S3" s="56">
         <f>R3*M3</f>
         <v>0.30449999999999999</v>
       </c>
-      <c r="T3" s="62"/>
+      <c r="T3" s="57"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
     </row>
@@ -2014,7 +2079,7 @@
       <c r="A4" s="33">
         <v>2</v>
       </c>
-      <c r="B4" s="54"/>
+      <c r="B4" s="99"/>
       <c r="C4" s="18" t="s">
         <v>35</v>
       </c>
@@ -2031,13 +2096,13 @@
         <v>39</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="K4" s="39">
         <v>7</v>
@@ -2049,8 +2114,8 @@
         <f t="shared" ref="M4:M39" si="0">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="63" t="s">
-        <v>196</v>
+      <c r="N4" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O4" s="40">
         <v>0.51580000000000004</v>
@@ -2063,7 +2128,7 @@
         <f t="shared" ref="Q4:Q39" si="2">O4*K4</f>
         <v>3.6106000000000003</v>
       </c>
-      <c r="R4" s="64">
+      <c r="R4" s="59">
         <v>0.51580000000000004</v>
       </c>
       <c r="S4" s="41">
@@ -2078,7 +2143,7 @@
       <c r="A5" s="33">
         <v>3</v>
       </c>
-      <c r="B5" s="54"/>
+      <c r="B5" s="99"/>
       <c r="C5" s="18" t="s">
         <v>40</v>
       </c>
@@ -2095,13 +2160,13 @@
         <v>43</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I5" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K5" s="39">
         <v>50</v>
@@ -2113,8 +2178,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N5" s="63" t="s">
-        <v>196</v>
+      <c r="N5" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O5" s="40">
         <v>6.6E-3</v>
@@ -2142,7 +2207,7 @@
       <c r="A6" s="33">
         <v>4</v>
       </c>
-      <c r="B6" s="54"/>
+      <c r="B6" s="99"/>
       <c r="C6" s="18" t="s">
         <v>44</v>
       </c>
@@ -2159,13 +2224,13 @@
         <v>43</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="I6" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K6" s="39">
         <v>100</v>
@@ -2177,10 +2242,10 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N6" s="65" t="s">
-        <v>196</v>
-      </c>
-      <c r="O6" s="72">
+      <c r="N6" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="O6" s="67">
         <v>2.8E-3</v>
       </c>
       <c r="P6" s="41">
@@ -2191,7 +2256,7 @@
         <f t="shared" si="2"/>
         <v>0.27999999999999997</v>
       </c>
-      <c r="R6" s="72">
+      <c r="R6" s="67">
         <v>2.8E-3</v>
       </c>
       <c r="S6" s="41">
@@ -2206,7 +2271,7 @@
       <c r="A7" s="33">
         <v>5</v>
       </c>
-      <c r="B7" s="54"/>
+      <c r="B7" s="99"/>
       <c r="C7" s="18" t="s">
         <v>47</v>
       </c>
@@ -2219,17 +2284,17 @@
       <c r="F7" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="70" t="s">
+      <c r="G7" s="65" t="s">
         <v>43</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="I7" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K7" s="39">
         <v>100</v>
@@ -2241,8 +2306,8 @@
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="N7" s="65" t="s">
-        <v>196</v>
+      <c r="N7" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O7" s="40">
         <v>7.6E-3</v>
@@ -2270,7 +2335,7 @@
       <c r="A8" s="33">
         <v>6</v>
       </c>
-      <c r="B8" s="54"/>
+      <c r="B8" s="99"/>
       <c r="C8" s="18" t="s">
         <v>50</v>
       </c>
@@ -2287,13 +2352,13 @@
         <v>54</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="I8" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="K8" s="39">
         <v>20</v>
@@ -2306,7 +2371,7 @@
         <v>10</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="O8" s="40">
         <v>2.87E-2</v>
@@ -2334,7 +2399,7 @@
       <c r="A9" s="33">
         <v>7</v>
       </c>
-      <c r="B9" s="54"/>
+      <c r="B9" s="99"/>
       <c r="C9" s="16" t="s">
         <v>55</v>
       </c>
@@ -2351,13 +2416,13 @@
         <v>43</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="I9" s="37" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K9" s="39">
         <v>50</v>
@@ -2369,10 +2434,10 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="N9" s="65" t="s">
-        <v>196</v>
-      </c>
-      <c r="O9" s="64">
+      <c r="N9" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="O9" s="59">
         <v>9.1000000000000004E-3</v>
       </c>
       <c r="P9" s="41">
@@ -2383,7 +2448,7 @@
         <f t="shared" si="2"/>
         <v>0.45500000000000002</v>
       </c>
-      <c r="R9" s="64">
+      <c r="R9" s="59">
         <v>9.1000000000000004E-3</v>
       </c>
       <c r="S9" s="41">
@@ -2398,7 +2463,7 @@
       <c r="A10" s="33">
         <v>8</v>
       </c>
-      <c r="B10" s="54"/>
+      <c r="B10" s="99"/>
       <c r="C10" s="18" t="s">
         <v>58</v>
       </c>
@@ -2411,17 +2476,17 @@
       <c r="F10" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="70" t="s">
+      <c r="G10" s="65" t="s">
         <v>61</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="I10" s="39" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="K10" s="39">
         <v>20</v>
@@ -2433,8 +2498,8 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N10" s="65" t="s">
-        <v>196</v>
+      <c r="N10" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O10" s="40">
         <v>3.7199999999999997E-2</v>
@@ -2447,7 +2512,7 @@
         <f t="shared" si="2"/>
         <v>0.74399999999999999</v>
       </c>
-      <c r="R10" s="64">
+      <c r="R10" s="59">
         <v>3.7199999999999997E-2</v>
       </c>
       <c r="S10" s="41">
@@ -2462,7 +2527,7 @@
       <c r="A11" s="33">
         <v>9</v>
       </c>
-      <c r="B11" s="54"/>
+      <c r="B11" s="99"/>
       <c r="C11" s="18" t="s">
         <v>62</v>
       </c>
@@ -2475,20 +2540,20 @@
       <c r="F11" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="G11" s="70" t="s">
-        <v>65</v>
+      <c r="G11" s="65" t="s">
+        <v>232</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>182</v>
+        <v>237</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>182</v>
+        <v>233</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="K11" s="39">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="L11" s="15">
         <v>2</v>
@@ -2497,26 +2562,25 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N11" s="65" t="s">
-        <v>207</v>
+      <c r="N11" s="106" t="s">
+        <v>192</v>
       </c>
       <c r="O11" s="40">
-        <v>0.14000000000000001</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="P11" s="41">
         <f t="shared" si="1"/>
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="Q11" s="41">
-        <f t="shared" si="2"/>
-        <v>2.8000000000000003</v>
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="Q11" s="40">
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="R11" s="40">
-        <v>0.14000000000000001</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="S11" s="41">
         <f t="shared" si="3"/>
-        <v>1.4000000000000001</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="T11" s="19"/>
       <c r="U11" s="3"/>
@@ -2526,43 +2590,43 @@
       <c r="A12" s="33">
         <v>10</v>
       </c>
-      <c r="B12" s="56"/>
-      <c r="C12" s="76" t="s">
+      <c r="B12" s="100"/>
+      <c r="C12" s="71" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="D12" s="74" t="s">
+      <c r="E12" s="69" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="74" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="74" t="s">
+      <c r="G12" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G12" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" s="66" t="s">
-        <v>208</v>
+      <c r="H12" s="61" t="s">
+        <v>203</v>
       </c>
       <c r="I12" s="46" t="s">
-        <v>182</v>
-      </c>
-      <c r="J12" s="74" t="s">
-        <v>181</v>
+        <v>178</v>
+      </c>
+      <c r="J12" s="69" t="s">
+        <v>177</v>
       </c>
       <c r="K12" s="45">
         <v>50</v>
       </c>
-      <c r="L12" s="75">
+      <c r="L12" s="70">
         <v>2</v>
       </c>
       <c r="M12" s="45">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N12" s="67" t="s">
-        <v>196</v>
+      <c r="N12" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="O12" s="42">
         <v>5.1000000000000004E-3</v>
@@ -2582,7 +2646,7 @@
         <f t="shared" si="3"/>
         <v>5.1000000000000004E-2</v>
       </c>
-      <c r="T12" s="68"/>
+      <c r="T12" s="63"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
     </row>
@@ -2590,55 +2654,63 @@
       <c r="A13" s="33">
         <v>11</v>
       </c>
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="98" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="E13" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="F13" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="G13" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="H13" s="50" t="s">
-        <v>182</v>
+        <v>236</v>
       </c>
       <c r="I13" s="48" t="s">
-        <v>182</v>
+        <v>234</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="K13" s="58"/>
-      <c r="L13" s="73">
+        <v>178</v>
+      </c>
+      <c r="K13" s="53">
+        <v>20</v>
+      </c>
+      <c r="L13" s="68">
         <v>4</v>
       </c>
-      <c r="M13" s="58">
+      <c r="M13" s="53">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N13" s="77"/>
-      <c r="O13" s="60"/>
-      <c r="P13" s="61">
+      <c r="N13" s="72" t="s">
+        <v>192</v>
+      </c>
+      <c r="O13" s="55">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="P13" s="56">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q13" s="61">
+        <v>6.9599999999999995E-2</v>
+      </c>
+      <c r="Q13" s="56">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R13" s="60"/>
-      <c r="S13" s="61">
+        <v>0.34799999999999998</v>
+      </c>
+      <c r="R13" s="55">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="S13" s="56">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.34799999999999998</v>
       </c>
       <c r="T13" s="12"/>
       <c r="U13" s="3"/>
@@ -2648,43 +2720,43 @@
       <c r="A14" s="33">
         <v>12</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="80" t="s">
+      <c r="B14" s="100"/>
+      <c r="C14" s="75" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="74" t="s">
+      <c r="E14" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="E14" s="74" t="s">
+      <c r="F14" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="F14" s="74" t="s">
+      <c r="G14" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H14" s="66" t="s">
-        <v>209</v>
+      <c r="H14" s="61" t="s">
+        <v>204</v>
       </c>
       <c r="I14" s="46" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K14" s="45">
         <v>12</v>
       </c>
-      <c r="L14" s="75">
+      <c r="L14" s="70">
         <v>2</v>
       </c>
       <c r="M14" s="45">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N14" s="67" t="s">
-        <v>196</v>
+      <c r="N14" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="O14" s="42">
         <v>0.97919999999999996</v>
@@ -2704,7 +2776,7 @@
         <f t="shared" si="3"/>
         <v>9.7919999999999998</v>
       </c>
-      <c r="T14" s="68"/>
+      <c r="T14" s="63"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
     </row>
@@ -2715,50 +2787,60 @@
       <c r="B15" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="78" t="s">
+        <v>241</v>
+      </c>
+      <c r="D15" s="79" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="79" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="79" t="s">
+        <v>242</v>
+      </c>
+      <c r="G15" s="80" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="85" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="85" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="85" t="s">
-        <v>82</v>
-      </c>
-      <c r="G15" s="86" t="s">
-        <v>83</v>
-      </c>
-      <c r="H15" s="87"/>
-      <c r="I15" s="88"/>
-      <c r="J15" s="85" t="s">
-        <v>183</v>
-      </c>
-      <c r="K15" s="89"/>
-      <c r="L15" s="90">
+      <c r="H15" s="81" t="s">
+        <v>243</v>
+      </c>
+      <c r="I15" s="82"/>
+      <c r="J15" s="79" t="s">
+        <v>179</v>
+      </c>
+      <c r="K15" s="83">
+        <v>7</v>
+      </c>
+      <c r="L15" s="84">
         <v>1</v>
       </c>
-      <c r="M15" s="89">
+      <c r="M15" s="83">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N15" s="91"/>
-      <c r="O15" s="92"/>
-      <c r="P15" s="93">
+      <c r="N15" s="108" t="s">
+        <v>192</v>
+      </c>
+      <c r="O15" s="85">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="P15" s="86">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="93">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="Q15" s="86">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R15" s="92"/>
-      <c r="S15" s="93">
+        <v>6.1585999999999999</v>
+      </c>
+      <c r="R15" s="85">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="S15" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="T15" s="107"/>
+        <v>4.399</v>
+      </c>
+      <c r="T15" s="97"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
     </row>
@@ -2766,65 +2848,65 @@
       <c r="A16" s="33">
         <v>14</v>
       </c>
-      <c r="B16" s="94" t="s">
+      <c r="B16" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="95" t="s">
+      <c r="C16" s="88" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="89" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" s="89" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="89" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="96" t="s">
+      <c r="G16" s="89" t="s">
         <v>85</v>
       </c>
-      <c r="E16" s="96" t="s">
-        <v>86</v>
-      </c>
-      <c r="F16" s="96" t="s">
-        <v>87</v>
-      </c>
-      <c r="G16" s="96" t="s">
-        <v>88</v>
-      </c>
-      <c r="H16" s="97" t="s">
-        <v>210</v>
-      </c>
-      <c r="I16" s="98" t="s">
-        <v>182</v>
-      </c>
-      <c r="J16" s="96" t="s">
-        <v>182</v>
-      </c>
-      <c r="K16" s="69">
+      <c r="H16" s="90" t="s">
+        <v>205</v>
+      </c>
+      <c r="I16" s="91" t="s">
+        <v>178</v>
+      </c>
+      <c r="J16" s="89" t="s">
+        <v>178</v>
+      </c>
+      <c r="K16" s="64">
         <v>10</v>
       </c>
-      <c r="L16" s="99">
+      <c r="L16" s="92">
         <v>1</v>
       </c>
-      <c r="M16" s="69">
+      <c r="M16" s="64">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N16" s="100" t="s">
-        <v>196</v>
-      </c>
-      <c r="O16" s="101">
+      <c r="N16" s="93" t="s">
+        <v>192</v>
+      </c>
+      <c r="O16" s="94">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="P16" s="102">
+      <c r="P16" s="95">
         <f t="shared" si="1"/>
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="Q16" s="102">
+      <c r="Q16" s="95">
         <f t="shared" si="2"/>
         <v>0.42999999999999994</v>
       </c>
-      <c r="R16" s="101">
+      <c r="R16" s="94">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="S16" s="102">
+      <c r="S16" s="95">
         <f t="shared" si="3"/>
         <v>0.21499999999999997</v>
       </c>
-      <c r="T16" s="103"/>
+      <c r="T16" s="96"/>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
     </row>
@@ -2832,65 +2914,65 @@
       <c r="A17" s="33">
         <v>15</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="98" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="G17" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="E17" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>93</v>
-      </c>
       <c r="H17" s="1" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="K17" s="58">
+        <v>180</v>
+      </c>
+      <c r="K17" s="53">
         <v>50</v>
       </c>
-      <c r="L17" s="73">
+      <c r="L17" s="68">
         <v>1</v>
       </c>
-      <c r="M17" s="58">
+      <c r="M17" s="53">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N17" s="77" t="s">
-        <v>196</v>
-      </c>
-      <c r="O17" s="60">
+      <c r="N17" s="72" t="s">
+        <v>192</v>
+      </c>
+      <c r="O17" s="55">
         <v>5.8999999999999999E-3</v>
       </c>
-      <c r="P17" s="61">
+      <c r="P17" s="56">
         <f t="shared" si="1"/>
         <v>5.8999999999999999E-3</v>
       </c>
-      <c r="Q17" s="61">
+      <c r="Q17" s="56">
         <f t="shared" si="2"/>
         <v>0.29499999999999998</v>
       </c>
-      <c r="R17" s="60">
+      <c r="R17" s="55">
         <v>5.8999999999999999E-3</v>
       </c>
-      <c r="S17" s="61">
+      <c r="S17" s="56">
         <f t="shared" si="3"/>
         <v>2.9499999999999998E-2</v>
       </c>
-      <c r="T17" s="78"/>
+      <c r="T17" s="73"/>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
     </row>
@@ -2898,30 +2980,30 @@
       <c r="A18" s="33">
         <v>16</v>
       </c>
-      <c r="B18" s="54"/>
+      <c r="B18" s="99"/>
       <c r="C18" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D18" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="F18" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="H18" s="51" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J18" s="17" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K18" s="39">
         <v>10</v>
@@ -2933,8 +3015,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N18" s="65" t="s">
-        <v>196</v>
+      <c r="N18" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O18" s="40">
         <v>6.7299999999999999E-2</v>
@@ -2962,30 +3044,30 @@
       <c r="A19" s="33">
         <v>17</v>
       </c>
-      <c r="B19" s="54"/>
+      <c r="B19" s="99"/>
       <c r="C19" s="18" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>43</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="I19" s="51" t="s">
+        <v>178</v>
+      </c>
+      <c r="J19" s="17" t="s">
         <v>182</v>
-      </c>
-      <c r="J19" s="17" t="s">
-        <v>186</v>
       </c>
       <c r="K19" s="39">
         <v>100</v>
@@ -2997,8 +3079,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="65" t="s">
-        <v>196</v>
+      <c r="N19" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O19" s="40">
         <v>2.3999999999999998E-3</v>
@@ -3026,30 +3108,30 @@
       <c r="A20" s="33">
         <v>18</v>
       </c>
-      <c r="B20" s="54"/>
+      <c r="B20" s="99"/>
       <c r="C20" s="18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>43</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="I20" s="51" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J20" s="17" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K20" s="39">
         <v>100</v>
@@ -3061,8 +3143,8 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N20" s="63" t="s">
-        <v>196</v>
+      <c r="N20" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O20" s="40">
         <v>1.4E-3</v>
@@ -3090,30 +3172,30 @@
       <c r="A21" s="33">
         <v>19</v>
       </c>
-      <c r="B21" s="54"/>
+      <c r="B21" s="99"/>
       <c r="C21" s="18" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="I21" s="37" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="J21" s="17" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="K21" s="39">
         <v>40</v>
@@ -3125,8 +3207,8 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N21" s="63" t="s">
-        <v>196</v>
+      <c r="N21" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O21" s="40">
         <v>3.9600000000000003E-2</v>
@@ -3146,8 +3228,8 @@
         <f t="shared" si="3"/>
         <v>0.79200000000000004</v>
       </c>
-      <c r="T21" s="79" t="s">
-        <v>234</v>
+      <c r="T21" s="74" t="s">
+        <v>229</v>
       </c>
       <c r="U21" s="3"/>
       <c r="V21" s="3"/>
@@ -3156,30 +3238,30 @@
       <c r="A22" s="33">
         <v>20</v>
       </c>
-      <c r="B22" s="54"/>
+      <c r="B22" s="99"/>
       <c r="C22" s="18" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>43</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="I22" s="51" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J22" s="17" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K22" s="39">
         <v>100</v>
@@ -3191,8 +3273,8 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N22" s="63" t="s">
-        <v>196</v>
+      <c r="N22" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O22" s="40">
         <v>1.4E-3</v>
@@ -3220,30 +3302,30 @@
       <c r="A23" s="33">
         <v>21</v>
       </c>
-      <c r="B23" s="54"/>
+      <c r="B23" s="99"/>
       <c r="C23" s="18" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>43</v>
       </c>
       <c r="H23" s="37" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J23" s="17" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K23" s="39">
         <v>50</v>
@@ -3255,8 +3337,8 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N23" s="65" t="s">
-        <v>196</v>
+      <c r="N23" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O23" s="40">
         <v>1.5800000000000002E-2</v>
@@ -3284,30 +3366,30 @@
       <c r="A24" s="33">
         <v>22</v>
       </c>
-      <c r="B24" s="54"/>
+      <c r="B24" s="99"/>
       <c r="C24" s="18" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>43</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J24" s="17" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="K24" s="5">
         <v>100</v>
@@ -3319,8 +3401,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="65" t="s">
-        <v>196</v>
+      <c r="N24" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O24" s="40">
         <v>1.9E-3</v>
@@ -3348,43 +3430,43 @@
       <c r="A25" s="33">
         <v>23</v>
       </c>
-      <c r="B25" s="56"/>
-      <c r="C25" s="76" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="74" t="s">
-        <v>117</v>
-      </c>
-      <c r="E25" s="74" t="s">
-        <v>91</v>
-      </c>
-      <c r="F25" s="74" t="s">
-        <v>118</v>
+      <c r="B25" s="100"/>
+      <c r="C25" s="71" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="69" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="69" t="s">
+        <v>88</v>
+      </c>
+      <c r="F25" s="69" t="s">
+        <v>115</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="H25" s="66" t="s">
-        <v>218</v>
+      <c r="H25" s="61" t="s">
+        <v>213</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="J25" s="74" t="s">
-        <v>192</v>
+        <v>178</v>
+      </c>
+      <c r="J25" s="69" t="s">
+        <v>188</v>
       </c>
       <c r="K25" s="8">
         <v>100</v>
       </c>
-      <c r="L25" s="75">
+      <c r="L25" s="70">
         <v>1</v>
       </c>
       <c r="M25" s="45">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N25" s="67" t="s">
-        <v>196</v>
+      <c r="N25" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="O25" s="42">
         <v>1.5E-3</v>
@@ -3404,7 +3486,7 @@
         <f t="shared" si="3"/>
         <v>7.4999999999999997E-3</v>
       </c>
-      <c r="T25" s="68"/>
+      <c r="T25" s="63"/>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
     </row>
@@ -3412,65 +3494,65 @@
       <c r="A26" s="33">
         <v>24</v>
       </c>
-      <c r="B26" s="55" t="s">
-        <v>197</v>
+      <c r="B26" s="98" t="s">
+        <v>193</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>52</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H26" s="50" t="s">
-        <v>182</v>
+        <v>235</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K26" s="1">
         <v>12</v>
       </c>
-      <c r="L26" s="73">
+      <c r="L26" s="68">
         <v>2</v>
       </c>
-      <c r="M26" s="58">
+      <c r="M26" s="53">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N26" s="77" t="s">
-        <v>207</v>
-      </c>
-      <c r="O26" s="60">
-        <v>0.55500000000000005</v>
-      </c>
-      <c r="P26" s="61">
+      <c r="N26" s="107" t="s">
+        <v>192</v>
+      </c>
+      <c r="O26" s="55">
+        <v>1.0188999999999999</v>
+      </c>
+      <c r="P26" s="56">
         <f t="shared" si="1"/>
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="Q26" s="61">
+        <v>2.0377999999999998</v>
+      </c>
+      <c r="Q26" s="56">
         <f t="shared" si="2"/>
-        <v>6.66</v>
-      </c>
-      <c r="R26" s="60">
-        <v>0.55500000000000005</v>
-      </c>
-      <c r="S26" s="61">
+        <v>12.226799999999999</v>
+      </c>
+      <c r="R26" s="55">
+        <v>0.79349999999999998</v>
+      </c>
+      <c r="S26" s="56">
         <f t="shared" si="3"/>
-        <v>5.5500000000000007</v>
-      </c>
-      <c r="T26" s="62"/>
+        <v>7.9349999999999996</v>
+      </c>
+      <c r="T26" s="57"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
     </row>
@@ -3478,43 +3560,43 @@
       <c r="A27" s="33">
         <v>25</v>
       </c>
-      <c r="B27" s="56"/>
-      <c r="C27" s="80" t="s">
-        <v>123</v>
+      <c r="B27" s="100"/>
+      <c r="C27" s="75" t="s">
+        <v>120</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="H27" s="66" t="s">
-        <v>220</v>
+        <v>214</v>
+      </c>
+      <c r="H27" s="61" t="s">
+        <v>215</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K27" s="8">
         <v>7</v>
       </c>
-      <c r="L27" s="75">
+      <c r="L27" s="70">
         <v>1</v>
       </c>
       <c r="M27" s="45">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="67" t="s">
-        <v>196</v>
+      <c r="N27" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="O27" s="42">
         <v>0.29239999999999999</v>
@@ -3534,7 +3616,7 @@
         <f t="shared" si="3"/>
         <v>1.462</v>
       </c>
-      <c r="T27" s="68"/>
+      <c r="T27" s="63"/>
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
     </row>
@@ -3542,65 +3624,65 @@
       <c r="A28" s="33">
         <v>26</v>
       </c>
-      <c r="B28" s="55" t="s">
-        <v>198</v>
-      </c>
-      <c r="C28" s="82" t="s">
-        <v>127</v>
+      <c r="B28" s="98" t="s">
+        <v>194</v>
+      </c>
+      <c r="C28" s="76" t="s">
+        <v>124</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>52</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="K28" s="1">
         <v>7</v>
       </c>
-      <c r="L28" s="73">
+      <c r="L28" s="68">
         <v>1</v>
       </c>
-      <c r="M28" s="58">
+      <c r="M28" s="53">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N28" s="77" t="s">
-        <v>196</v>
-      </c>
-      <c r="O28" s="60">
+      <c r="N28" s="72" t="s">
+        <v>192</v>
+      </c>
+      <c r="O28" s="55">
         <v>0.49590000000000001</v>
       </c>
-      <c r="P28" s="61">
+      <c r="P28" s="56">
         <f t="shared" si="1"/>
         <v>0.49590000000000001</v>
       </c>
-      <c r="Q28" s="61">
+      <c r="Q28" s="56">
         <f t="shared" si="2"/>
         <v>3.4713000000000003</v>
       </c>
-      <c r="R28" s="60">
+      <c r="R28" s="55">
         <v>0.49590000000000001</v>
       </c>
-      <c r="S28" s="61">
+      <c r="S28" s="56">
         <f t="shared" si="3"/>
         <v>2.4794999999999998</v>
       </c>
-      <c r="T28" s="62"/>
+      <c r="T28" s="57"/>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
     </row>
@@ -3608,43 +3690,43 @@
       <c r="A29" s="33">
         <v>27</v>
       </c>
-      <c r="B29" s="56"/>
-      <c r="C29" s="80" t="s">
+      <c r="B29" s="100"/>
+      <c r="C29" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="D29" s="69" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="69" t="s">
+        <v>52</v>
+      </c>
+      <c r="F29" s="69" t="s">
+        <v>129</v>
+      </c>
+      <c r="G29" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="D29" s="74" t="s">
-        <v>131</v>
-      </c>
-      <c r="E29" s="74" t="s">
-        <v>52</v>
-      </c>
-      <c r="F29" s="74" t="s">
-        <v>132</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="H29" s="66" t="s">
-        <v>222</v>
+      <c r="H29" s="61" t="s">
+        <v>217</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K29" s="8">
         <v>7</v>
       </c>
-      <c r="L29" s="75">
+      <c r="L29" s="70">
         <v>1</v>
       </c>
       <c r="M29" s="45">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N29" s="67" t="s">
-        <v>196</v>
+      <c r="N29" s="62" t="s">
+        <v>192</v>
       </c>
       <c r="O29" s="42">
         <v>0.4148</v>
@@ -3664,7 +3746,7 @@
         <f t="shared" si="3"/>
         <v>2.0739999999999998</v>
       </c>
-      <c r="T29" s="68"/>
+      <c r="T29" s="63"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
     </row>
@@ -3672,65 +3754,65 @@
       <c r="A30" s="33">
         <v>28</v>
       </c>
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="98" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="F30" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="G30" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E30" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="H30" s="50" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="I30" s="50" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K30" s="1">
         <v>6</v>
       </c>
-      <c r="L30" s="73">
+      <c r="L30" s="68">
         <v>1</v>
       </c>
-      <c r="M30" s="58">
+      <c r="M30" s="53">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N30" s="77" t="s">
-        <v>196</v>
-      </c>
-      <c r="O30" s="60">
+      <c r="N30" s="72" t="s">
+        <v>192</v>
+      </c>
+      <c r="O30" s="55">
         <v>3.9186000000000001</v>
       </c>
-      <c r="P30" s="61">
+      <c r="P30" s="56">
         <f t="shared" si="1"/>
         <v>3.9186000000000001</v>
       </c>
-      <c r="Q30" s="61">
+      <c r="Q30" s="56">
         <f t="shared" si="2"/>
         <v>23.511600000000001</v>
       </c>
-      <c r="R30" s="60">
+      <c r="R30" s="55">
         <v>3.9186000000000001</v>
       </c>
-      <c r="S30" s="61">
+      <c r="S30" s="56">
         <f t="shared" si="3"/>
         <v>19.593</v>
       </c>
-      <c r="T30" s="62"/>
+      <c r="T30" s="57"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
     </row>
@@ -3738,30 +3820,30 @@
       <c r="A31" s="33">
         <v>29</v>
       </c>
-      <c r="B31" s="54"/>
+      <c r="B31" s="99"/>
       <c r="C31" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D31" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="H31" s="37" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="I31" s="37" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K31" s="39">
         <v>6</v>
@@ -3773,8 +3855,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N31" s="63" t="s">
-        <v>196</v>
+      <c r="N31" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O31" s="40">
         <v>15.131399999999999</v>
@@ -3802,30 +3884,30 @@
       <c r="A32" s="33">
         <v>30</v>
       </c>
-      <c r="B32" s="54"/>
+      <c r="B32" s="99"/>
       <c r="C32" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="F32" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="D32" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="F32" s="17" t="s">
-        <v>146</v>
-      </c>
       <c r="G32" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H32" s="37" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="I32" s="38" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K32" s="39">
         <v>6</v>
@@ -3837,8 +3919,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N32" s="63" t="s">
-        <v>196</v>
+      <c r="N32" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O32" s="40">
         <v>0.30049999999999999</v>
@@ -3866,30 +3948,30 @@
       <c r="A33" s="33">
         <v>31</v>
       </c>
-      <c r="B33" s="54"/>
+      <c r="B33" s="99"/>
       <c r="C33" s="16" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H33" s="37" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="I33" s="51" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K33" s="39">
         <v>6</v>
@@ -3901,8 +3983,8 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N33" s="63" t="s">
-        <v>196</v>
+      <c r="N33" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O33" s="40">
         <v>0.32629999999999998</v>
@@ -3930,30 +4012,30 @@
       <c r="A34" s="33">
         <v>32</v>
       </c>
-      <c r="B34" s="54"/>
+      <c r="B34" s="99"/>
       <c r="C34" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="F34" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="D34" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>154</v>
-      </c>
       <c r="G34" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H34" s="37" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K34" s="39">
         <v>6</v>
@@ -3965,8 +4047,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N34" s="63" t="s">
-        <v>196</v>
+      <c r="N34" s="58" t="s">
+        <v>192</v>
       </c>
       <c r="O34" s="40">
         <v>1.3868</v>
@@ -3994,51 +4076,53 @@
       <c r="A35" s="33">
         <v>33</v>
       </c>
-      <c r="B35" s="56"/>
-      <c r="C35" s="80" t="s">
+      <c r="B35" s="100"/>
+      <c r="C35" s="119" t="s">
+        <v>152</v>
+      </c>
+      <c r="D35" s="109" t="s">
+        <v>153</v>
+      </c>
+      <c r="E35" s="110" t="s">
+        <v>154</v>
+      </c>
+      <c r="F35" s="109" t="s">
         <v>155</v>
       </c>
-      <c r="D35" s="74" t="s">
+      <c r="G35" s="111" t="s">
         <v>156</v>
       </c>
-      <c r="E35" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="F35" s="74" t="s">
-        <v>158</v>
-      </c>
-      <c r="G35" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="H35" s="66"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="K35" s="45"/>
-      <c r="L35" s="75">
+      <c r="H35" s="112"/>
+      <c r="I35" s="111"/>
+      <c r="J35" s="111" t="s">
+        <v>178</v>
+      </c>
+      <c r="K35" s="113"/>
+      <c r="L35" s="114">
         <v>5</v>
       </c>
-      <c r="M35" s="45">
+      <c r="M35" s="113">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N35" s="81"/>
-      <c r="O35" s="42"/>
-      <c r="P35" s="43">
+      <c r="N35" s="115"/>
+      <c r="O35" s="116"/>
+      <c r="P35" s="117">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q35" s="43">
+      <c r="Q35" s="117">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="R35" s="42"/>
-      <c r="S35" s="43">
+      <c r="R35" s="116"/>
+      <c r="S35" s="117">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="T35" s="68"/>
+      <c r="T35" s="118" t="s">
+        <v>238</v>
+      </c>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
     </row>
@@ -4046,65 +4130,65 @@
       <c r="A36" s="33">
         <v>34</v>
       </c>
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="98" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>52</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H36" s="50" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="K36" s="58">
+        <v>178</v>
+      </c>
+      <c r="K36" s="53">
         <v>30</v>
       </c>
-      <c r="L36" s="73">
+      <c r="L36" s="68">
         <v>5</v>
       </c>
-      <c r="M36" s="58">
+      <c r="M36" s="53">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N36" s="77" t="s">
-        <v>196</v>
-      </c>
-      <c r="O36" s="83">
+      <c r="N36" s="72" t="s">
+        <v>192</v>
+      </c>
+      <c r="O36" s="77">
         <v>9.8900000000000002E-2</v>
       </c>
-      <c r="P36" s="61">
+      <c r="P36" s="56">
         <f t="shared" si="1"/>
         <v>0.4945</v>
       </c>
-      <c r="Q36" s="61">
+      <c r="Q36" s="56">
         <f t="shared" si="2"/>
         <v>2.9670000000000001</v>
       </c>
-      <c r="R36" s="83">
+      <c r="R36" s="77">
         <v>9.8900000000000002E-2</v>
       </c>
-      <c r="S36" s="61">
+      <c r="S36" s="56">
         <f t="shared" si="3"/>
         <v>2.4725000000000001</v>
       </c>
-      <c r="T36" s="78"/>
+      <c r="T36" s="73"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
     </row>
@@ -4112,30 +4196,30 @@
       <c r="A37" s="33">
         <v>35</v>
       </c>
-      <c r="B37" s="54"/>
+      <c r="B37" s="99"/>
       <c r="C37" s="18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E37" s="17" t="s">
         <v>52</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="H37" s="37" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K37" s="39">
         <v>7</v>
@@ -4147,8 +4231,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N37" s="65" t="s">
-        <v>196</v>
+      <c r="N37" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="O37" s="40">
         <v>0.27289999999999998</v>
@@ -4174,28 +4258,32 @@
       <c r="A38" s="33">
         <v>36</v>
       </c>
-      <c r="B38" s="54"/>
+      <c r="B38" s="99"/>
       <c r="C38" s="18" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E38" s="17" t="s">
         <v>52</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="H38" s="37"/>
+        <v>165</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>239</v>
+      </c>
       <c r="I38" s="5"/>
       <c r="J38" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="K38" s="39"/>
+        <v>191</v>
+      </c>
+      <c r="K38" s="39">
+        <v>7</v>
+      </c>
       <c r="L38" s="15">
         <v>1</v>
       </c>
@@ -4203,20 +4291,26 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N38" s="65"/>
-      <c r="O38" s="40"/>
+      <c r="N38" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="O38" s="40">
+        <v>0.1804</v>
+      </c>
       <c r="P38" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1804</v>
       </c>
       <c r="Q38" s="41">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R38" s="40"/>
+        <v>1.2627999999999999</v>
+      </c>
+      <c r="R38" s="40">
+        <v>0.14430000000000001</v>
+      </c>
       <c r="S38" s="41">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.72150000000000003</v>
       </c>
       <c r="T38" s="49"/>
       <c r="U38" s="3"/>
@@ -4226,43 +4320,43 @@
       <c r="A39" s="33">
         <v>37</v>
       </c>
-      <c r="B39" s="56"/>
-      <c r="C39" s="76" t="s">
-        <v>170</v>
-      </c>
-      <c r="D39" s="74" t="s">
-        <v>171</v>
-      </c>
-      <c r="E39" s="74" t="s">
+      <c r="B39" s="100"/>
+      <c r="C39" s="71" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="69" t="s">
+        <v>167</v>
+      </c>
+      <c r="E39" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="F39" s="74" t="s">
-        <v>172</v>
+      <c r="F39" s="69" t="s">
+        <v>168</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="H39" s="66" t="s">
-        <v>236</v>
+        <v>165</v>
+      </c>
+      <c r="H39" s="61" t="s">
+        <v>231</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K39" s="45">
         <v>7</v>
       </c>
-      <c r="L39" s="75">
+      <c r="L39" s="70">
         <v>1</v>
       </c>
       <c r="M39" s="45">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N39" s="71" t="s">
-        <v>196</v>
+      <c r="N39" s="66" t="s">
+        <v>192</v>
       </c>
       <c r="O39" s="42">
         <v>0.22420000000000001</v>
@@ -4291,21 +4385,21 @@
       <c r="I40" s="26"/>
       <c r="J40" s="26"/>
       <c r="K40" s="26"/>
-      <c r="L40" s="57" t="s">
+      <c r="L40" s="105" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="57"/>
-      <c r="N40" s="57"/>
-      <c r="O40" s="57"/>
+      <c r="M40" s="105"/>
+      <c r="N40" s="105"/>
+      <c r="O40" s="105"/>
       <c r="P40" s="30"/>
       <c r="Q40" s="30">
         <f>SUM(Q3:Q39)</f>
-        <v>174.70999999999998</v>
+        <v>185.24939999999998</v>
       </c>
       <c r="R40" s="30"/>
       <c r="S40" s="22">
         <f>SUM(S3:S39)</f>
-        <v>142.85650000000001</v>
+        <v>149.34200000000001</v>
       </c>
       <c r="T40" s="26"/>
       <c r="U40" s="3"/>
@@ -4316,21 +4410,21 @@
       <c r="I41" s="26"/>
       <c r="J41" s="28"/>
       <c r="K41" s="26"/>
-      <c r="L41" s="53" t="s">
+      <c r="L41" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="53"/>
-      <c r="N41" s="53"/>
-      <c r="O41" s="53"/>
+      <c r="M41" s="101"/>
+      <c r="N41" s="101"/>
+      <c r="O41" s="101"/>
       <c r="P41" s="22">
         <f>SUM(P3:P39)</f>
-        <v>28.844199999999997</v>
+        <v>30.628199999999996</v>
       </c>
       <c r="Q41" s="22"/>
       <c r="R41" s="27"/>
       <c r="S41" s="29">
         <f>S40/5</f>
-        <v>28.571300000000001</v>
+        <v>29.868400000000001</v>
       </c>
       <c r="T41" s="26"/>
       <c r="U41" s="3"/>
@@ -4554,7 +4648,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:Q39">
+  <conditionalFormatting sqref="P3:Q10 P12:Q39 P11">
     <cfRule type="dataBar" priority="42">
       <dataBar>
         <cfvo type="min"/>
@@ -4583,42 +4677,44 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N8" r:id="rId1"/>
-    <hyperlink ref="N3" r:id="rId2"/>
-    <hyperlink ref="N4" r:id="rId3"/>
-    <hyperlink ref="N5" r:id="rId4"/>
-    <hyperlink ref="N6" r:id="rId5"/>
-    <hyperlink ref="N7" r:id="rId6"/>
-    <hyperlink ref="N9" r:id="rId7"/>
-    <hyperlink ref="N10" r:id="rId8"/>
-    <hyperlink ref="N11" r:id="rId9"/>
-    <hyperlink ref="N12" r:id="rId10"/>
-    <hyperlink ref="N14" r:id="rId11"/>
-    <hyperlink ref="N16" r:id="rId12"/>
-    <hyperlink ref="N17" r:id="rId13"/>
-    <hyperlink ref="N18" r:id="rId14"/>
-    <hyperlink ref="N19" r:id="rId15"/>
-    <hyperlink ref="N20" r:id="rId16"/>
-    <hyperlink ref="N22" r:id="rId17"/>
-    <hyperlink ref="N23" r:id="rId18"/>
-    <hyperlink ref="N24" r:id="rId19"/>
-    <hyperlink ref="N25" r:id="rId20"/>
-    <hyperlink ref="N26" r:id="rId21"/>
-    <hyperlink ref="N27" r:id="rId22"/>
-    <hyperlink ref="N28" r:id="rId23"/>
-    <hyperlink ref="N29" r:id="rId24"/>
-    <hyperlink ref="N30" r:id="rId25"/>
-    <hyperlink ref="N31" r:id="rId26"/>
-    <hyperlink ref="N32" r:id="rId27"/>
-    <hyperlink ref="N33" r:id="rId28"/>
-    <hyperlink ref="N34" r:id="rId29"/>
-    <hyperlink ref="N36" r:id="rId30"/>
-    <hyperlink ref="N37" r:id="rId31"/>
-    <hyperlink ref="N21" r:id="rId32"/>
-    <hyperlink ref="N39" r:id="rId33"/>
+    <hyperlink ref="N8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N17" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N32" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="N33" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="N34" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="N36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="N37" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="N21" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="N39" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N11" r:id="rId33" xr:uid="{625CBE1A-0F89-4C4C-A1FE-B24967D4F28E}"/>
+    <hyperlink ref="N13" r:id="rId34" xr:uid="{884106D0-4856-4ED0-8613-7AF2716041FF}"/>
+    <hyperlink ref="N15" r:id="rId35" xr:uid="{D92F47DE-DF6F-4DD6-B73D-E984E3B960F3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId34"/>
+  <pageSetup orientation="portrait" r:id="rId36"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -4711,7 +4807,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:Q39</xm:sqref>
+          <xm:sqref>P3:Q10 P12:Q39 P11</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C84B8479-0C38-4E8A-A10C-CE0A75F3F79C}">

</xml_diff>

<commit_message>
power switch link and price added to LCSC BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SaleemD-CustomProduct\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4727EBDF-5191-4006-BA8F-66D32420769B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,7 +18,7 @@
   <definedNames>
     <definedName name="LCSC">Sheet1!$N$20</definedName>
   </definedNames>
-  <calcPr calcId="162913" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="242">
   <si>
     <t>S. No.</t>
   </si>
@@ -741,9 +742,6 @@
     <t>C106245</t>
   </si>
   <si>
-    <t>Awaiting reponse of custom supplier</t>
-  </si>
-  <si>
     <t>C125616</t>
   </si>
   <si>
@@ -767,12 +765,15 @@
   </si>
   <si>
     <t>Bill of Material (BOM) for Saleem Custom Product</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -894,7 +895,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -915,12 +916,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1284,7 +1279,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1350,16 +1345,16 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1573,38 +1568,29 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="21" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1630,29 +1616,14 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1934,7 +1905,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1960,28 +1931,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="115" t="s">
-        <v>241</v>
-      </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="117"/>
+      <c r="A1" s="112" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="I1" s="113"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="113"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="113"/>
+      <c r="O1" s="113"/>
+      <c r="P1" s="113"/>
+      <c r="Q1" s="113"/>
+      <c r="R1" s="113"/>
+      <c r="S1" s="113"/>
+      <c r="T1" s="114"/>
     </row>
     <row r="2" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
@@ -2049,13 +2020,13 @@
       <c r="A3" s="33">
         <v>1</v>
       </c>
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="108" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="122" t="s">
+      <c r="D3" s="103" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="14" t="s">
@@ -2115,11 +2086,11 @@
       <c r="A4" s="33">
         <v>2</v>
       </c>
-      <c r="B4" s="112"/>
+      <c r="B4" s="109"/>
       <c r="C4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="123" t="s">
+      <c r="D4" s="104" t="s">
         <v>35</v>
       </c>
       <c r="E4" s="17" t="s">
@@ -2179,11 +2150,11 @@
       <c r="A5" s="33">
         <v>3</v>
       </c>
-      <c r="B5" s="112"/>
+      <c r="B5" s="109"/>
       <c r="C5" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="123" t="s">
+      <c r="D5" s="104" t="s">
         <v>40</v>
       </c>
       <c r="E5" s="17" t="s">
@@ -2243,11 +2214,11 @@
       <c r="A6" s="33">
         <v>4</v>
       </c>
-      <c r="B6" s="112"/>
+      <c r="B6" s="109"/>
       <c r="C6" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="123" t="s">
+      <c r="D6" s="104" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="17" t="s">
@@ -2307,11 +2278,11 @@
       <c r="A7" s="33">
         <v>5</v>
       </c>
-      <c r="B7" s="112"/>
+      <c r="B7" s="109"/>
       <c r="C7" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="123" t="s">
+      <c r="D7" s="104" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="17" t="s">
@@ -2371,11 +2342,11 @@
       <c r="A8" s="33">
         <v>6</v>
       </c>
-      <c r="B8" s="112"/>
+      <c r="B8" s="109"/>
       <c r="C8" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="123" t="s">
+      <c r="D8" s="104" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="17" t="s">
@@ -2435,7 +2406,7 @@
       <c r="A9" s="33">
         <v>7</v>
       </c>
-      <c r="B9" s="112"/>
+      <c r="B9" s="109"/>
       <c r="C9" s="16" t="s">
         <v>54</v>
       </c>
@@ -2499,17 +2470,17 @@
       <c r="A10" s="33">
         <v>8</v>
       </c>
-      <c r="B10" s="112"/>
+      <c r="B10" s="109"/>
       <c r="C10" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="123" t="s">
+      <c r="D10" s="104" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="120" t="s">
+      <c r="F10" s="101" t="s">
         <v>59</v>
       </c>
       <c r="G10" s="64" t="s">
@@ -2563,17 +2534,17 @@
       <c r="A11" s="33">
         <v>9</v>
       </c>
-      <c r="B11" s="112"/>
+      <c r="B11" s="109"/>
       <c r="C11" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="123" t="s">
+      <c r="D11" s="104" t="s">
         <v>62</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="121" t="s">
+      <c r="F11" s="102" t="s">
         <v>63</v>
       </c>
       <c r="G11" s="64" t="s">
@@ -2626,11 +2597,11 @@
       <c r="A12" s="33">
         <v>10</v>
       </c>
-      <c r="B12" s="113"/>
+      <c r="B12" s="110"/>
       <c r="C12" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="124" t="s">
+      <c r="D12" s="105" t="s">
         <v>65</v>
       </c>
       <c r="E12" s="68" t="s">
@@ -2690,19 +2661,19 @@
       <c r="A13" s="33">
         <v>11</v>
       </c>
-      <c r="B13" s="111" t="s">
+      <c r="B13" s="108" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="122" t="s">
+      <c r="D13" s="103" t="s">
         <v>69</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="119" t="s">
+      <c r="F13" s="100" t="s">
         <v>71</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -2756,11 +2727,11 @@
       <c r="A14" s="33">
         <v>12</v>
       </c>
-      <c r="B14" s="113"/>
+      <c r="B14" s="110"/>
       <c r="C14" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="124" t="s">
+      <c r="D14" s="105" t="s">
         <v>74</v>
       </c>
       <c r="E14" s="68" t="s">
@@ -2824,22 +2795,22 @@
         <v>20</v>
       </c>
       <c r="C15" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="D15" s="125" t="s">
+        <v>235</v>
+      </c>
+      <c r="D15" s="106" t="s">
         <v>78</v>
       </c>
       <c r="E15" s="77" t="s">
         <v>51</v>
       </c>
       <c r="F15" s="77" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G15" s="78" t="s">
         <v>79</v>
       </c>
       <c r="H15" s="79" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I15" s="80"/>
       <c r="J15" s="77" t="s">
@@ -2890,7 +2861,7 @@
       <c r="C16" s="86" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="126" t="s">
+      <c r="D16" s="107" t="s">
         <v>81</v>
       </c>
       <c r="E16" s="87" t="s">
@@ -2950,13 +2921,13 @@
       <c r="A17" s="33">
         <v>15</v>
       </c>
-      <c r="B17" s="111" t="s">
+      <c r="B17" s="108" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="122" t="s">
+      <c r="D17" s="103" t="s">
         <v>86</v>
       </c>
       <c r="E17" s="14" t="s">
@@ -3016,11 +2987,11 @@
       <c r="A18" s="33">
         <v>16</v>
       </c>
-      <c r="B18" s="112"/>
+      <c r="B18" s="109"/>
       <c r="C18" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="123" t="s">
+      <c r="D18" s="104" t="s">
         <v>91</v>
       </c>
       <c r="E18" s="17" t="s">
@@ -3080,11 +3051,11 @@
       <c r="A19" s="33">
         <v>17</v>
       </c>
-      <c r="B19" s="112"/>
+      <c r="B19" s="109"/>
       <c r="C19" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="123" t="s">
+      <c r="D19" s="104" t="s">
         <v>95</v>
       </c>
       <c r="E19" s="17" t="s">
@@ -3144,11 +3115,11 @@
       <c r="A20" s="33">
         <v>18</v>
       </c>
-      <c r="B20" s="112"/>
+      <c r="B20" s="109"/>
       <c r="C20" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="123" t="s">
+      <c r="D20" s="104" t="s">
         <v>98</v>
       </c>
       <c r="E20" s="17" t="s">
@@ -3208,15 +3179,15 @@
       <c r="A21" s="33">
         <v>19</v>
       </c>
-      <c r="B21" s="112"/>
+      <c r="B21" s="109"/>
       <c r="C21" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D21" s="38" t="s">
         <v>100</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>223</v>
@@ -3272,11 +3243,11 @@
       <c r="A22" s="33">
         <v>20</v>
       </c>
-      <c r="B22" s="112"/>
+      <c r="B22" s="109"/>
       <c r="C22" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="123" t="s">
+      <c r="D22" s="104" t="s">
         <v>102</v>
       </c>
       <c r="E22" s="17" t="s">
@@ -3336,11 +3307,11 @@
       <c r="A23" s="33">
         <v>21</v>
       </c>
-      <c r="B23" s="112"/>
+      <c r="B23" s="109"/>
       <c r="C23" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="123" t="s">
+      <c r="D23" s="104" t="s">
         <v>105</v>
       </c>
       <c r="E23" s="17" t="s">
@@ -3400,11 +3371,11 @@
       <c r="A24" s="33">
         <v>22</v>
       </c>
-      <c r="B24" s="112"/>
+      <c r="B24" s="109"/>
       <c r="C24" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D24" s="123" t="s">
+      <c r="D24" s="104" t="s">
         <v>108</v>
       </c>
       <c r="E24" s="17" t="s">
@@ -3464,11 +3435,11 @@
       <c r="A25" s="33">
         <v>23</v>
       </c>
-      <c r="B25" s="113"/>
+      <c r="B25" s="110"/>
       <c r="C25" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="124" t="s">
+      <c r="D25" s="105" t="s">
         <v>111</v>
       </c>
       <c r="E25" s="68" t="s">
@@ -3528,7 +3499,7 @@
       <c r="A26" s="33">
         <v>24</v>
       </c>
-      <c r="B26" s="111" t="s">
+      <c r="B26" s="108" t="s">
         <v>190</v>
       </c>
       <c r="C26" s="13" t="s">
@@ -3594,7 +3565,7 @@
       <c r="A27" s="33">
         <v>25</v>
       </c>
-      <c r="B27" s="113"/>
+      <c r="B27" s="110"/>
       <c r="C27" s="73" t="s">
         <v>117</v>
       </c>
@@ -3658,7 +3629,7 @@
       <c r="A28" s="33">
         <v>26</v>
       </c>
-      <c r="B28" s="111" t="s">
+      <c r="B28" s="108" t="s">
         <v>191</v>
       </c>
       <c r="C28" s="74" t="s">
@@ -3724,7 +3695,7 @@
       <c r="A29" s="33">
         <v>27</v>
       </c>
-      <c r="B29" s="113"/>
+      <c r="B29" s="110"/>
       <c r="C29" s="73" t="s">
         <v>124</v>
       </c>
@@ -3788,7 +3759,7 @@
       <c r="A30" s="33">
         <v>28</v>
       </c>
-      <c r="B30" s="111" t="s">
+      <c r="B30" s="108" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="13" t="s">
@@ -3854,7 +3825,7 @@
       <c r="A31" s="33">
         <v>29</v>
       </c>
-      <c r="B31" s="112"/>
+      <c r="B31" s="109"/>
       <c r="C31" s="18" t="s">
         <v>133</v>
       </c>
@@ -3918,7 +3889,7 @@
       <c r="A32" s="33">
         <v>30</v>
       </c>
-      <c r="B32" s="112"/>
+      <c r="B32" s="109"/>
       <c r="C32" s="18" t="s">
         <v>137</v>
       </c>
@@ -3982,7 +3953,7 @@
       <c r="A33" s="33">
         <v>31</v>
       </c>
-      <c r="B33" s="112"/>
+      <c r="B33" s="109"/>
       <c r="C33" s="16" t="s">
         <v>141</v>
       </c>
@@ -4008,7 +3979,7 @@
         <v>175</v>
       </c>
       <c r="K33" s="39">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="L33" s="15">
         <v>4</v>
@@ -4029,7 +4000,7 @@
       </c>
       <c r="Q33" s="41">
         <f t="shared" si="2"/>
-        <v>1.9577999999999998</v>
+        <v>8.1574999999999989</v>
       </c>
       <c r="R33" s="40">
         <v>0.32629999999999998</v>
@@ -4046,7 +4017,7 @@
       <c r="A34" s="33">
         <v>32</v>
       </c>
-      <c r="B34" s="112"/>
+      <c r="B34" s="109"/>
       <c r="C34" s="18" t="s">
         <v>145</v>
       </c>
@@ -4110,53 +4081,63 @@
       <c r="A35" s="33">
         <v>33</v>
       </c>
-      <c r="B35" s="113"/>
-      <c r="C35" s="110" t="s">
+      <c r="B35" s="110"/>
+      <c r="C35" s="116" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="100" t="s">
+      <c r="D35" s="105" t="s">
         <v>150</v>
       </c>
-      <c r="E35" s="101" t="s">
+      <c r="E35" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="F35" s="100" t="s">
+      <c r="F35" s="105" t="s">
         <v>152</v>
       </c>
-      <c r="G35" s="102" t="s">
+      <c r="G35" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="H35" s="103"/>
-      <c r="I35" s="102"/>
-      <c r="J35" s="102" t="s">
+      <c r="H35" s="60" t="s">
         <v>175</v>
       </c>
-      <c r="K35" s="104"/>
-      <c r="L35" s="105">
+      <c r="I35" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="K35" s="45">
+        <v>30</v>
+      </c>
+      <c r="L35" s="117">
         <v>5</v>
       </c>
-      <c r="M35" s="104">
+      <c r="M35" s="45">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N35" s="106"/>
-      <c r="O35" s="107"/>
-      <c r="P35" s="108">
+      <c r="N35" s="118" t="s">
+        <v>241</v>
+      </c>
+      <c r="O35" s="42">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="P35" s="43">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q35" s="108">
+        <v>2.31</v>
+      </c>
+      <c r="Q35" s="43">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R35" s="107"/>
-      <c r="S35" s="108">
+        <v>13.860000000000001</v>
+      </c>
+      <c r="R35" s="42">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="S35" s="43">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="T35" s="109" t="s">
-        <v>233</v>
-      </c>
+        <v>11.55</v>
+      </c>
+      <c r="T35" s="62"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
     </row>
@@ -4164,7 +4145,7 @@
       <c r="A36" s="33">
         <v>34</v>
       </c>
-      <c r="B36" s="111" t="s">
+      <c r="B36" s="108" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="13" t="s">
@@ -4230,7 +4211,7 @@
       <c r="A37" s="33">
         <v>35</v>
       </c>
-      <c r="B37" s="112"/>
+      <c r="B37" s="109"/>
       <c r="C37" s="18" t="s">
         <v>157</v>
       </c>
@@ -4294,7 +4275,7 @@
       <c r="A38" s="33">
         <v>36</v>
       </c>
-      <c r="B38" s="112"/>
+      <c r="B38" s="109"/>
       <c r="C38" s="18" t="s">
         <v>160</v>
       </c>
@@ -4305,13 +4286,13 @@
         <v>51</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G38" s="4" t="s">
         <v>162</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="4" t="s">
@@ -4356,7 +4337,7 @@
       <c r="A39" s="33">
         <v>37</v>
       </c>
-      <c r="B39" s="113"/>
+      <c r="B39" s="110"/>
       <c r="C39" s="70" t="s">
         <v>163</v>
       </c>
@@ -4421,21 +4402,21 @@
       <c r="I40" s="26"/>
       <c r="J40" s="26"/>
       <c r="K40" s="26"/>
-      <c r="L40" s="118" t="s">
+      <c r="L40" s="115" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="118"/>
-      <c r="N40" s="118"/>
-      <c r="O40" s="118"/>
+      <c r="M40" s="115"/>
+      <c r="N40" s="115"/>
+      <c r="O40" s="115"/>
       <c r="P40" s="30"/>
       <c r="Q40" s="30">
         <f>SUM(Q3:Q39)</f>
-        <v>185.59739999999999</v>
+        <v>205.65710000000001</v>
       </c>
       <c r="R40" s="30"/>
       <c r="S40" s="22">
         <f>SUM(S3:S39)</f>
-        <v>150.70650000000001</v>
+        <v>162.25650000000002</v>
       </c>
       <c r="T40" s="26"/>
       <c r="U40" s="3"/>
@@ -4446,24 +4427,24 @@
       <c r="I41" s="26"/>
       <c r="J41" s="28"/>
       <c r="K41" s="26"/>
-      <c r="L41" s="114" t="s">
+      <c r="L41" s="111" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="114"/>
-      <c r="N41" s="114"/>
-      <c r="O41" s="114"/>
+      <c r="M41" s="111"/>
+      <c r="N41" s="111"/>
+      <c r="O41" s="111"/>
       <c r="P41" s="22">
         <f>SUM(P3:P39)</f>
-        <v>30.628199999999996</v>
+        <v>32.938200000000002</v>
       </c>
       <c r="Q41" s="22">
         <f>Q40/5</f>
-        <v>37.119479999999996</v>
+        <v>41.131420000000006</v>
       </c>
       <c r="R41" s="27"/>
       <c r="S41" s="29">
         <f>S40/5</f>
-        <v>30.141300000000001</v>
+        <v>32.451300000000003</v>
       </c>
       <c r="T41" s="26"/>
       <c r="U41" s="3"/>
@@ -4716,44 +4697,45 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N8" r:id="rId1"/>
-    <hyperlink ref="N3" r:id="rId2"/>
-    <hyperlink ref="N4" r:id="rId3"/>
-    <hyperlink ref="N5" r:id="rId4"/>
-    <hyperlink ref="N6" r:id="rId5"/>
-    <hyperlink ref="N7" r:id="rId6"/>
-    <hyperlink ref="N9" r:id="rId7"/>
-    <hyperlink ref="N10" r:id="rId8"/>
-    <hyperlink ref="N12" r:id="rId9"/>
-    <hyperlink ref="N14" r:id="rId10"/>
-    <hyperlink ref="N16" r:id="rId11"/>
-    <hyperlink ref="N17" r:id="rId12"/>
-    <hyperlink ref="N18" r:id="rId13"/>
-    <hyperlink ref="N19" r:id="rId14"/>
-    <hyperlink ref="N20" r:id="rId15"/>
-    <hyperlink ref="N22" r:id="rId16"/>
-    <hyperlink ref="N23" r:id="rId17"/>
-    <hyperlink ref="N24" r:id="rId18"/>
-    <hyperlink ref="N25" r:id="rId19"/>
-    <hyperlink ref="N26" r:id="rId20"/>
-    <hyperlink ref="N27" r:id="rId21"/>
-    <hyperlink ref="N28" r:id="rId22"/>
-    <hyperlink ref="N29" r:id="rId23"/>
-    <hyperlink ref="N30" r:id="rId24"/>
-    <hyperlink ref="N31" r:id="rId25"/>
-    <hyperlink ref="N32" r:id="rId26"/>
-    <hyperlink ref="N33" r:id="rId27"/>
-    <hyperlink ref="N34" r:id="rId28"/>
-    <hyperlink ref="N36" r:id="rId29"/>
-    <hyperlink ref="N37" r:id="rId30"/>
-    <hyperlink ref="N21" r:id="rId31"/>
-    <hyperlink ref="N39" r:id="rId32"/>
-    <hyperlink ref="N11" r:id="rId33"/>
-    <hyperlink ref="N13" r:id="rId34"/>
-    <hyperlink ref="N15" r:id="rId35"/>
+    <hyperlink ref="N8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N17" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N32" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N33" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="N34" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="N36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="N37" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="N21" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="N39" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="N11" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N13" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="N15" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="N35" r:id="rId36" xr:uid="{22803AA7-377B-442D-B7F9-22DAF87C6ADB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId36"/>
+  <pageSetup orientation="portrait" r:id="rId37"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Fabrication BOM Add kia ha  LCSC BOM ki price Change hui ha Digikey BOM me alternate part add howe han
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24430"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4727EBDF-5191-4006-BA8F-66D32420769B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="LCSC">Sheet1!$N$20</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -773,7 +772,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1279,7 +1278,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1556,9 +1555,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1592,6 +1588,21 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1615,15 +1626,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1905,7 +1907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1931,28 +1933,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="116" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
-      <c r="O1" s="113"/>
-      <c r="P1" s="113"/>
-      <c r="Q1" s="113"/>
-      <c r="R1" s="113"/>
-      <c r="S1" s="113"/>
-      <c r="T1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="118"/>
     </row>
     <row r="2" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
@@ -2020,13 +2022,13 @@
       <c r="A3" s="33">
         <v>1</v>
       </c>
-      <c r="B3" s="108" t="s">
+      <c r="B3" s="112" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="103" t="s">
+      <c r="D3" s="102" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="14" t="s">
@@ -2086,11 +2088,11 @@
       <c r="A4" s="33">
         <v>2</v>
       </c>
-      <c r="B4" s="109"/>
+      <c r="B4" s="113"/>
       <c r="C4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="104" t="s">
+      <c r="D4" s="103" t="s">
         <v>35</v>
       </c>
       <c r="E4" s="17" t="s">
@@ -2125,22 +2127,22 @@
         <v>189</v>
       </c>
       <c r="O4" s="40">
-        <v>0.51580000000000004</v>
+        <v>0.55730000000000002</v>
       </c>
       <c r="P4" s="41">
         <f t="shared" ref="P4:P39" si="1">O4*L4</f>
-        <v>0.51580000000000004</v>
+        <v>0.55730000000000002</v>
       </c>
       <c r="Q4" s="41">
         <f t="shared" ref="Q4:Q39" si="2">O4*K4</f>
-        <v>3.6106000000000003</v>
+        <v>3.9011</v>
       </c>
       <c r="R4" s="58">
-        <v>0.51580000000000004</v>
+        <v>0.55730000000000002</v>
       </c>
       <c r="S4" s="41">
         <f t="shared" ref="S4:S39" si="3">R4*M4</f>
-        <v>2.5790000000000002</v>
+        <v>2.7865000000000002</v>
       </c>
       <c r="T4" s="49"/>
       <c r="U4" s="3"/>
@@ -2150,11 +2152,11 @@
       <c r="A5" s="33">
         <v>3</v>
       </c>
-      <c r="B5" s="109"/>
+      <c r="B5" s="113"/>
       <c r="C5" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="104" t="s">
+      <c r="D5" s="103" t="s">
         <v>40</v>
       </c>
       <c r="E5" s="17" t="s">
@@ -2189,22 +2191,22 @@
         <v>189</v>
       </c>
       <c r="O5" s="40">
-        <v>6.6E-3</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="P5" s="41">
         <f t="shared" si="1"/>
-        <v>6.6E-3</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="Q5" s="41">
         <f t="shared" si="2"/>
-        <v>0.33</v>
+        <v>0.30499999999999999</v>
       </c>
       <c r="R5" s="40">
-        <v>6.6E-3</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="S5" s="41">
         <f t="shared" si="3"/>
-        <v>3.3000000000000002E-2</v>
+        <v>3.0500000000000003E-2</v>
       </c>
       <c r="T5" s="49"/>
       <c r="U5" s="3"/>
@@ -2214,11 +2216,11 @@
       <c r="A6" s="33">
         <v>4</v>
       </c>
-      <c r="B6" s="109"/>
+      <c r="B6" s="113"/>
       <c r="C6" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="104" t="s">
+      <c r="D6" s="103" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="17" t="s">
@@ -2278,11 +2280,11 @@
       <c r="A7" s="33">
         <v>5</v>
       </c>
-      <c r="B7" s="109"/>
+      <c r="B7" s="113"/>
       <c r="C7" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="104" t="s">
+      <c r="D7" s="103" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="17" t="s">
@@ -2317,22 +2319,22 @@
         <v>189</v>
       </c>
       <c r="O7" s="40">
-        <v>7.6E-3</v>
+        <v>8.2000000000000007E-3</v>
       </c>
       <c r="P7" s="41">
         <f t="shared" si="1"/>
-        <v>0.10639999999999999</v>
+        <v>0.11480000000000001</v>
       </c>
       <c r="Q7" s="41">
         <f t="shared" si="2"/>
-        <v>0.76</v>
+        <v>0.82000000000000006</v>
       </c>
       <c r="R7" s="40">
-        <v>7.6E-3</v>
+        <v>8.2000000000000007E-3</v>
       </c>
       <c r="S7" s="41">
         <f t="shared" si="3"/>
-        <v>0.53200000000000003</v>
+        <v>0.57400000000000007</v>
       </c>
       <c r="T7" s="19"/>
       <c r="U7" s="3"/>
@@ -2342,11 +2344,11 @@
       <c r="A8" s="33">
         <v>6</v>
       </c>
-      <c r="B8" s="109"/>
+      <c r="B8" s="113"/>
       <c r="C8" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="104" t="s">
+      <c r="D8" s="103" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="17" t="s">
@@ -2381,22 +2383,22 @@
         <v>189</v>
       </c>
       <c r="O8" s="40">
-        <v>2.87E-2</v>
+        <v>2.98E-2</v>
       </c>
       <c r="P8" s="41">
         <f t="shared" si="1"/>
-        <v>5.74E-2</v>
+        <v>5.96E-2</v>
       </c>
       <c r="Q8" s="41">
         <f t="shared" si="2"/>
-        <v>0.57399999999999995</v>
+        <v>0.59599999999999997</v>
       </c>
       <c r="R8" s="40">
-        <v>2.87E-2</v>
+        <v>2.98E-2</v>
       </c>
       <c r="S8" s="41">
         <f t="shared" si="3"/>
-        <v>0.28699999999999998</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="T8" s="49"/>
       <c r="U8" s="3"/>
@@ -2406,7 +2408,7 @@
       <c r="A9" s="33">
         <v>7</v>
       </c>
-      <c r="B9" s="109"/>
+      <c r="B9" s="113"/>
       <c r="C9" s="16" t="s">
         <v>54</v>
       </c>
@@ -2445,22 +2447,22 @@
         <v>189</v>
       </c>
       <c r="O9" s="58">
-        <v>9.1000000000000004E-3</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="P9" s="41">
         <f t="shared" si="1"/>
-        <v>6.3700000000000007E-2</v>
+        <v>7.1400000000000005E-2</v>
       </c>
       <c r="Q9" s="41">
         <f t="shared" si="2"/>
-        <v>0.45500000000000002</v>
+        <v>0.51</v>
       </c>
       <c r="R9" s="58">
-        <v>9.1000000000000004E-3</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="S9" s="41">
         <f t="shared" si="3"/>
-        <v>0.31850000000000001</v>
+        <v>0.35700000000000004</v>
       </c>
       <c r="T9" s="49"/>
       <c r="U9" s="3"/>
@@ -2470,17 +2472,17 @@
       <c r="A10" s="33">
         <v>8</v>
       </c>
-      <c r="B10" s="109"/>
+      <c r="B10" s="113"/>
       <c r="C10" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="104" t="s">
+      <c r="D10" s="103" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="101" t="s">
+      <c r="F10" s="100" t="s">
         <v>59</v>
       </c>
       <c r="G10" s="64" t="s">
@@ -2509,22 +2511,22 @@
         <v>189</v>
       </c>
       <c r="O10" s="40">
-        <v>3.7199999999999997E-2</v>
+        <v>3.5400000000000001E-2</v>
       </c>
       <c r="P10" s="41">
         <f t="shared" si="1"/>
-        <v>7.4399999999999994E-2</v>
+        <v>7.0800000000000002E-2</v>
       </c>
       <c r="Q10" s="41">
         <f t="shared" si="2"/>
-        <v>0.74399999999999999</v>
+        <v>0.70799999999999996</v>
       </c>
       <c r="R10" s="58">
-        <v>3.7199999999999997E-2</v>
+        <v>3.5400000000000001E-2</v>
       </c>
       <c r="S10" s="41">
         <f t="shared" si="3"/>
-        <v>0.372</v>
+        <v>0.35399999999999998</v>
       </c>
       <c r="T10" s="19"/>
       <c r="U10" s="3"/>
@@ -2534,17 +2536,17 @@
       <c r="A11" s="33">
         <v>9</v>
       </c>
-      <c r="B11" s="109"/>
+      <c r="B11" s="113"/>
       <c r="C11" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="104" t="s">
+      <c r="D11" s="103" t="s">
         <v>62</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="102" t="s">
+      <c r="F11" s="101" t="s">
         <v>63</v>
       </c>
       <c r="G11" s="64" t="s">
@@ -2560,7 +2562,7 @@
         <v>173</v>
       </c>
       <c r="K11" s="39">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="L11" s="15">
         <v>2</v>
@@ -2569,25 +2571,25 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N11" s="97" t="s">
+      <c r="N11" s="96" t="s">
         <v>189</v>
       </c>
       <c r="O11" s="40">
-        <v>3.2000000000000002E-3</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="P11" s="41">
         <f t="shared" si="1"/>
-        <v>6.4000000000000003E-3</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="Q11" s="40">
         <v>3.2000000000000002E-3</v>
       </c>
       <c r="R11" s="40">
-        <v>3.2000000000000002E-3</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="S11" s="41">
         <f t="shared" si="3"/>
-        <v>3.2000000000000001E-2</v>
+        <v>0.03</v>
       </c>
       <c r="T11" s="19"/>
       <c r="U11" s="3"/>
@@ -2597,11 +2599,11 @@
       <c r="A12" s="33">
         <v>10</v>
       </c>
-      <c r="B12" s="110"/>
+      <c r="B12" s="114"/>
       <c r="C12" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="105" t="s">
+      <c r="D12" s="104" t="s">
         <v>65</v>
       </c>
       <c r="E12" s="68" t="s">
@@ -2661,19 +2663,19 @@
       <c r="A13" s="33">
         <v>11</v>
       </c>
-      <c r="B13" s="108" t="s">
+      <c r="B13" s="112" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="103" t="s">
+      <c r="D13" s="102" t="s">
         <v>69</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="100" t="s">
+      <c r="F13" s="99" t="s">
         <v>71</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -2727,11 +2729,11 @@
       <c r="A14" s="33">
         <v>12</v>
       </c>
-      <c r="B14" s="110"/>
+      <c r="B14" s="114"/>
       <c r="C14" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="105" t="s">
+      <c r="D14" s="104" t="s">
         <v>74</v>
       </c>
       <c r="E14" s="68" t="s">
@@ -2766,22 +2768,22 @@
         <v>189</v>
       </c>
       <c r="O14" s="42">
-        <v>0.97919999999999996</v>
+        <v>0.93589999999999995</v>
       </c>
       <c r="P14" s="43">
         <f t="shared" si="1"/>
-        <v>1.9583999999999999</v>
+        <v>1.8717999999999999</v>
       </c>
       <c r="Q14" s="43">
         <f t="shared" si="2"/>
-        <v>11.750399999999999</v>
+        <v>11.230799999999999</v>
       </c>
       <c r="R14" s="42">
-        <v>0.97919999999999996</v>
+        <v>0.69069999999999998</v>
       </c>
       <c r="S14" s="43">
         <f t="shared" si="3"/>
-        <v>9.7919999999999998</v>
+        <v>6.907</v>
       </c>
       <c r="T14" s="62"/>
       <c r="U14" s="3"/>
@@ -2791,13 +2793,13 @@
       <c r="A15" s="33">
         <v>13</v>
       </c>
-      <c r="B15" s="96" t="s">
+      <c r="B15" s="110" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>235</v>
       </c>
-      <c r="D15" s="106" t="s">
+      <c r="D15" s="105" t="s">
         <v>78</v>
       </c>
       <c r="E15" s="77" t="s">
@@ -2826,7 +2828,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N15" s="99" t="s">
+      <c r="N15" s="98" t="s">
         <v>189</v>
       </c>
       <c r="O15" s="83">
@@ -2861,7 +2863,7 @@
       <c r="C16" s="86" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="107" t="s">
+      <c r="D16" s="106" t="s">
         <v>81</v>
       </c>
       <c r="E16" s="87" t="s">
@@ -2883,7 +2885,7 @@
         <v>175</v>
       </c>
       <c r="K16" s="63">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L16" s="90">
         <v>1</v>
@@ -2896,22 +2898,22 @@
         <v>189</v>
       </c>
       <c r="O16" s="92">
-        <v>4.2999999999999997E-2</v>
+        <v>4.07E-2</v>
       </c>
       <c r="P16" s="93">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.07E-2</v>
       </c>
       <c r="Q16" s="93">
         <f t="shared" si="2"/>
-        <v>0.42999999999999994</v>
+        <v>0.81400000000000006</v>
       </c>
       <c r="R16" s="92">
-        <v>4.2999999999999997E-2</v>
+        <v>4.07E-2</v>
       </c>
       <c r="S16" s="93">
         <f t="shared" si="3"/>
-        <v>0.21499999999999997</v>
+        <v>0.20350000000000001</v>
       </c>
       <c r="T16" s="94"/>
       <c r="U16" s="3"/>
@@ -2921,13 +2923,13 @@
       <c r="A17" s="33">
         <v>15</v>
       </c>
-      <c r="B17" s="108" t="s">
+      <c r="B17" s="112" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="103" t="s">
+      <c r="D17" s="102" t="s">
         <v>86</v>
       </c>
       <c r="E17" s="14" t="s">
@@ -2962,22 +2964,22 @@
         <v>189</v>
       </c>
       <c r="O17" s="54">
-        <v>5.8999999999999999E-3</v>
+        <v>1.8E-3</v>
       </c>
       <c r="P17" s="55">
         <f t="shared" si="1"/>
-        <v>5.8999999999999999E-3</v>
+        <v>1.8E-3</v>
       </c>
       <c r="Q17" s="55">
         <f t="shared" si="2"/>
-        <v>0.29499999999999998</v>
+        <v>0.09</v>
       </c>
       <c r="R17" s="54">
-        <v>5.8999999999999999E-3</v>
+        <v>1.8E-3</v>
       </c>
       <c r="S17" s="55">
         <f t="shared" si="3"/>
-        <v>2.9499999999999998E-2</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="T17" s="72"/>
       <c r="U17" s="3"/>
@@ -2987,11 +2989,11 @@
       <c r="A18" s="33">
         <v>16</v>
       </c>
-      <c r="B18" s="109"/>
+      <c r="B18" s="113"/>
       <c r="C18" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="104" t="s">
+      <c r="D18" s="103" t="s">
         <v>91</v>
       </c>
       <c r="E18" s="17" t="s">
@@ -3026,22 +3028,22 @@
         <v>189</v>
       </c>
       <c r="O18" s="40">
-        <v>6.7299999999999999E-2</v>
+        <v>6.0699999999999997E-2</v>
       </c>
       <c r="P18" s="41">
         <f t="shared" si="1"/>
-        <v>6.7299999999999999E-2</v>
+        <v>6.0699999999999997E-2</v>
       </c>
       <c r="Q18" s="41">
         <f t="shared" si="2"/>
-        <v>0.67300000000000004</v>
+        <v>0.60699999999999998</v>
       </c>
       <c r="R18" s="40">
-        <v>6.7299999999999999E-2</v>
+        <v>6.0699999999999997E-2</v>
       </c>
       <c r="S18" s="41">
         <f t="shared" si="3"/>
-        <v>0.33650000000000002</v>
+        <v>0.30349999999999999</v>
       </c>
       <c r="T18" s="20"/>
       <c r="U18" s="3"/>
@@ -3051,11 +3053,11 @@
       <c r="A19" s="33">
         <v>17</v>
       </c>
-      <c r="B19" s="109"/>
+      <c r="B19" s="113"/>
       <c r="C19" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="104" t="s">
+      <c r="D19" s="103" t="s">
         <v>95</v>
       </c>
       <c r="E19" s="17" t="s">
@@ -3115,11 +3117,11 @@
       <c r="A20" s="33">
         <v>18</v>
       </c>
-      <c r="B20" s="109"/>
+      <c r="B20" s="113"/>
       <c r="C20" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="104" t="s">
+      <c r="D20" s="103" t="s">
         <v>98</v>
       </c>
       <c r="E20" s="17" t="s">
@@ -3179,7 +3181,7 @@
       <c r="A21" s="33">
         <v>19</v>
       </c>
-      <c r="B21" s="109"/>
+      <c r="B21" s="113"/>
       <c r="C21" s="16" t="s">
         <v>238</v>
       </c>
@@ -3218,22 +3220,22 @@
         <v>189</v>
       </c>
       <c r="O21" s="40">
-        <v>3.9600000000000003E-2</v>
+        <v>3.7600000000000001E-2</v>
       </c>
       <c r="P21" s="41">
         <f t="shared" si="1"/>
-        <v>0.15840000000000001</v>
+        <v>0.15040000000000001</v>
       </c>
       <c r="Q21" s="41">
         <f t="shared" si="2"/>
-        <v>1.5840000000000001</v>
+        <v>1.504</v>
       </c>
       <c r="R21" s="40">
-        <v>3.9600000000000003E-2</v>
+        <v>3.7600000000000001E-2</v>
       </c>
       <c r="S21" s="41">
         <f t="shared" si="3"/>
-        <v>0.79200000000000004</v>
+        <v>0.752</v>
       </c>
       <c r="T21" s="49"/>
       <c r="U21" s="3"/>
@@ -3243,11 +3245,11 @@
       <c r="A22" s="33">
         <v>20</v>
       </c>
-      <c r="B22" s="109"/>
+      <c r="B22" s="113"/>
       <c r="C22" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="104" t="s">
+      <c r="D22" s="103" t="s">
         <v>102</v>
       </c>
       <c r="E22" s="17" t="s">
@@ -3282,22 +3284,22 @@
         <v>189</v>
       </c>
       <c r="O22" s="40">
-        <v>1.4E-3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="P22" s="41">
         <f t="shared" si="1"/>
-        <v>5.5999999999999999E-3</v>
+        <v>6.7999999999999996E-3</v>
       </c>
       <c r="Q22" s="41">
         <f t="shared" si="2"/>
-        <v>0.13999999999999999</v>
+        <v>0.16999999999999998</v>
       </c>
       <c r="R22" s="40">
-        <v>1.4E-3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="S22" s="41">
         <f t="shared" si="3"/>
-        <v>2.8000000000000001E-2</v>
+        <v>3.3999999999999996E-2</v>
       </c>
       <c r="T22" s="49"/>
       <c r="U22" s="3"/>
@@ -3307,11 +3309,11 @@
       <c r="A23" s="33">
         <v>21</v>
       </c>
-      <c r="B23" s="109"/>
+      <c r="B23" s="113"/>
       <c r="C23" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="104" t="s">
+      <c r="D23" s="103" t="s">
         <v>105</v>
       </c>
       <c r="E23" s="17" t="s">
@@ -3346,22 +3348,22 @@
         <v>189</v>
       </c>
       <c r="O23" s="40">
-        <v>1.5800000000000002E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="P23" s="41">
         <f t="shared" si="1"/>
-        <v>6.3200000000000006E-2</v>
+        <v>0.06</v>
       </c>
       <c r="Q23" s="41">
         <f t="shared" si="2"/>
-        <v>0.79</v>
+        <v>0.75</v>
       </c>
       <c r="R23" s="40">
-        <v>1.5800000000000002E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="S23" s="41">
         <f t="shared" si="3"/>
-        <v>0.31600000000000006</v>
+        <v>0.3</v>
       </c>
       <c r="T23" s="49"/>
       <c r="U23" s="3"/>
@@ -3371,11 +3373,11 @@
       <c r="A24" s="33">
         <v>22</v>
       </c>
-      <c r="B24" s="109"/>
+      <c r="B24" s="113"/>
       <c r="C24" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D24" s="104" t="s">
+      <c r="D24" s="103" t="s">
         <v>108</v>
       </c>
       <c r="E24" s="17" t="s">
@@ -3410,22 +3412,22 @@
         <v>189</v>
       </c>
       <c r="O24" s="40">
-        <v>1.9E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="P24" s="41">
         <f t="shared" si="1"/>
-        <v>1.9E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="Q24" s="41">
         <f t="shared" si="2"/>
-        <v>0.19</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="R24" s="40">
-        <v>1.9E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="S24" s="41">
         <f t="shared" si="3"/>
-        <v>9.4999999999999998E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="T24" s="49"/>
       <c r="U24" s="3"/>
@@ -3435,11 +3437,11 @@
       <c r="A25" s="33">
         <v>23</v>
       </c>
-      <c r="B25" s="110"/>
+      <c r="B25" s="114"/>
       <c r="C25" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="105" t="s">
+      <c r="D25" s="104" t="s">
         <v>111</v>
       </c>
       <c r="E25" s="68" t="s">
@@ -3499,7 +3501,7 @@
       <c r="A26" s="33">
         <v>24</v>
       </c>
-      <c r="B26" s="108" t="s">
+      <c r="B26" s="112" t="s">
         <v>190</v>
       </c>
       <c r="C26" s="13" t="s">
@@ -3536,26 +3538,26 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N26" s="98" t="s">
+      <c r="N26" s="97" t="s">
         <v>189</v>
       </c>
       <c r="O26" s="54">
-        <v>1.0188999999999999</v>
+        <v>0.88370000000000004</v>
       </c>
       <c r="P26" s="55">
         <f t="shared" si="1"/>
-        <v>2.0377999999999998</v>
+        <v>1.7674000000000001</v>
       </c>
       <c r="Q26" s="55">
         <f t="shared" si="2"/>
-        <v>12.226799999999999</v>
+        <v>10.6044</v>
       </c>
       <c r="R26" s="54">
-        <v>0.79349999999999998</v>
+        <v>0.65820000000000001</v>
       </c>
       <c r="S26" s="55">
         <f t="shared" si="3"/>
-        <v>7.9349999999999996</v>
+        <v>6.5819999999999999</v>
       </c>
       <c r="T26" s="56"/>
       <c r="U26" s="3"/>
@@ -3565,7 +3567,7 @@
       <c r="A27" s="33">
         <v>25</v>
       </c>
-      <c r="B27" s="110"/>
+      <c r="B27" s="114"/>
       <c r="C27" s="73" t="s">
         <v>117</v>
       </c>
@@ -3604,22 +3606,22 @@
         <v>189</v>
       </c>
       <c r="O27" s="42">
-        <v>0.29239999999999999</v>
+        <v>0.28449999999999998</v>
       </c>
       <c r="P27" s="43">
         <f t="shared" si="1"/>
-        <v>0.29239999999999999</v>
+        <v>0.28449999999999998</v>
       </c>
       <c r="Q27" s="43">
         <f t="shared" si="2"/>
-        <v>2.0468000000000002</v>
+        <v>1.9914999999999998</v>
       </c>
       <c r="R27" s="42">
-        <v>0.29239999999999999</v>
+        <v>0.28449999999999998</v>
       </c>
       <c r="S27" s="43">
         <f t="shared" si="3"/>
-        <v>1.462</v>
+        <v>1.4224999999999999</v>
       </c>
       <c r="T27" s="62"/>
       <c r="U27" s="3"/>
@@ -3629,7 +3631,7 @@
       <c r="A28" s="33">
         <v>26</v>
       </c>
-      <c r="B28" s="108" t="s">
+      <c r="B28" s="112" t="s">
         <v>191</v>
       </c>
       <c r="C28" s="74" t="s">
@@ -3695,7 +3697,7 @@
       <c r="A29" s="33">
         <v>27</v>
       </c>
-      <c r="B29" s="110"/>
+      <c r="B29" s="114"/>
       <c r="C29" s="73" t="s">
         <v>124</v>
       </c>
@@ -3734,22 +3736,22 @@
         <v>189</v>
       </c>
       <c r="O29" s="42">
-        <v>0.4148</v>
+        <v>0.41120000000000001</v>
       </c>
       <c r="P29" s="43">
         <f t="shared" si="1"/>
-        <v>0.4148</v>
+        <v>0.41120000000000001</v>
       </c>
       <c r="Q29" s="43">
         <f t="shared" si="2"/>
-        <v>2.9036</v>
+        <v>2.8784000000000001</v>
       </c>
       <c r="R29" s="42">
-        <v>0.4148</v>
+        <v>0.41120000000000001</v>
       </c>
       <c r="S29" s="43">
         <f t="shared" si="3"/>
-        <v>2.0739999999999998</v>
+        <v>2.056</v>
       </c>
       <c r="T29" s="62"/>
       <c r="U29" s="3"/>
@@ -3759,7 +3761,7 @@
       <c r="A30" s="33">
         <v>28</v>
       </c>
-      <c r="B30" s="108" t="s">
+      <c r="B30" s="112" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="13" t="s">
@@ -3800,22 +3802,22 @@
         <v>189</v>
       </c>
       <c r="O30" s="54">
-        <v>3.9186000000000001</v>
+        <v>3.8355999999999999</v>
       </c>
       <c r="P30" s="55">
         <f t="shared" si="1"/>
-        <v>3.9186000000000001</v>
+        <v>3.8355999999999999</v>
       </c>
       <c r="Q30" s="55">
         <f t="shared" si="2"/>
-        <v>23.511600000000001</v>
+        <v>23.0136</v>
       </c>
       <c r="R30" s="54">
-        <v>3.9186000000000001</v>
+        <v>3.8355999999999999</v>
       </c>
       <c r="S30" s="55">
         <f t="shared" si="3"/>
-        <v>19.593</v>
+        <v>19.178000000000001</v>
       </c>
       <c r="T30" s="56"/>
       <c r="U30" s="3"/>
@@ -3825,7 +3827,7 @@
       <c r="A31" s="33">
         <v>29</v>
       </c>
-      <c r="B31" s="109"/>
+      <c r="B31" s="113"/>
       <c r="C31" s="18" t="s">
         <v>133</v>
       </c>
@@ -3889,7 +3891,7 @@
       <c r="A32" s="33">
         <v>30</v>
       </c>
-      <c r="B32" s="109"/>
+      <c r="B32" s="113"/>
       <c r="C32" s="18" t="s">
         <v>137</v>
       </c>
@@ -3953,7 +3955,7 @@
       <c r="A33" s="33">
         <v>31</v>
       </c>
-      <c r="B33" s="109"/>
+      <c r="B33" s="113"/>
       <c r="C33" s="16" t="s">
         <v>141</v>
       </c>
@@ -3992,22 +3994,22 @@
         <v>189</v>
       </c>
       <c r="O33" s="40">
-        <v>0.32629999999999998</v>
+        <v>0.26579999999999998</v>
       </c>
       <c r="P33" s="41">
         <f t="shared" si="1"/>
-        <v>1.3051999999999999</v>
+        <v>1.0631999999999999</v>
       </c>
       <c r="Q33" s="41">
         <f t="shared" si="2"/>
-        <v>8.1574999999999989</v>
+        <v>6.6449999999999996</v>
       </c>
       <c r="R33" s="40">
-        <v>0.32629999999999998</v>
+        <v>0.26579999999999998</v>
       </c>
       <c r="S33" s="41">
         <f t="shared" si="3"/>
-        <v>6.5259999999999998</v>
+        <v>5.3159999999999998</v>
       </c>
       <c r="T33" s="49"/>
       <c r="U33" s="3"/>
@@ -4017,7 +4019,7 @@
       <c r="A34" s="33">
         <v>32</v>
       </c>
-      <c r="B34" s="109"/>
+      <c r="B34" s="113"/>
       <c r="C34" s="18" t="s">
         <v>145</v>
       </c>
@@ -4056,22 +4058,22 @@
         <v>189</v>
       </c>
       <c r="O34" s="40">
-        <v>1.3868</v>
+        <v>1.0964</v>
       </c>
       <c r="P34" s="41">
         <f t="shared" si="1"/>
-        <v>1.3868</v>
+        <v>1.0964</v>
       </c>
       <c r="Q34" s="41">
         <f t="shared" si="2"/>
-        <v>8.3208000000000002</v>
+        <v>6.5784000000000002</v>
       </c>
       <c r="R34" s="40">
-        <v>1.3868</v>
+        <v>1.0964</v>
       </c>
       <c r="S34" s="41">
         <f t="shared" si="3"/>
-        <v>6.9340000000000002</v>
+        <v>5.4820000000000002</v>
       </c>
       <c r="T34" s="49"/>
       <c r="U34" s="3"/>
@@ -4081,17 +4083,17 @@
       <c r="A35" s="33">
         <v>33</v>
       </c>
-      <c r="B35" s="110"/>
-      <c r="C35" s="116" t="s">
+      <c r="B35" s="114"/>
+      <c r="C35" s="107" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="105" t="s">
+      <c r="D35" s="104" t="s">
         <v>150</v>
       </c>
       <c r="E35" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="F35" s="105" t="s">
+      <c r="F35" s="104" t="s">
         <v>152</v>
       </c>
       <c r="G35" s="8" t="s">
@@ -4109,14 +4111,14 @@
       <c r="K35" s="45">
         <v>30</v>
       </c>
-      <c r="L35" s="117">
+      <c r="L35" s="108">
         <v>5</v>
       </c>
       <c r="M35" s="45">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N35" s="118" t="s">
+      <c r="N35" s="109" t="s">
         <v>241</v>
       </c>
       <c r="O35" s="42">
@@ -4145,7 +4147,7 @@
       <c r="A36" s="33">
         <v>34</v>
       </c>
-      <c r="B36" s="108" t="s">
+      <c r="B36" s="112" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="13" t="s">
@@ -4186,22 +4188,22 @@
         <v>189</v>
       </c>
       <c r="O36" s="75">
-        <v>9.8900000000000002E-2</v>
+        <v>9.2399999999999996E-2</v>
       </c>
       <c r="P36" s="55">
         <f t="shared" si="1"/>
-        <v>0.4945</v>
+        <v>0.46199999999999997</v>
       </c>
       <c r="Q36" s="55">
         <f t="shared" si="2"/>
-        <v>2.9670000000000001</v>
+        <v>2.7719999999999998</v>
       </c>
       <c r="R36" s="75">
-        <v>9.8900000000000002E-2</v>
+        <v>9.2399999999999996E-2</v>
       </c>
       <c r="S36" s="55">
         <f t="shared" si="3"/>
-        <v>2.4725000000000001</v>
+        <v>2.31</v>
       </c>
       <c r="T36" s="72"/>
       <c r="U36" s="3"/>
@@ -4211,7 +4213,7 @@
       <c r="A37" s="33">
         <v>35</v>
       </c>
-      <c r="B37" s="109"/>
+      <c r="B37" s="113"/>
       <c r="C37" s="18" t="s">
         <v>157</v>
       </c>
@@ -4250,22 +4252,22 @@
         <v>189</v>
       </c>
       <c r="O37" s="40">
-        <v>0.27289999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="P37" s="41">
         <f t="shared" si="1"/>
-        <v>0.27289999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="Q37" s="41">
         <f t="shared" si="2"/>
-        <v>1.9102999999999999</v>
+        <v>1.75</v>
       </c>
       <c r="R37" s="40">
-        <v>0.27289999999999998</v>
+        <v>0.25</v>
       </c>
       <c r="S37" s="41">
         <f t="shared" si="3"/>
-        <v>1.3644999999999998</v>
+        <v>1.25</v>
       </c>
       <c r="T37" s="49"/>
       <c r="U37" s="3"/>
@@ -4275,7 +4277,7 @@
       <c r="A38" s="33">
         <v>36</v>
       </c>
-      <c r="B38" s="109"/>
+      <c r="B38" s="113"/>
       <c r="C38" s="18" t="s">
         <v>160</v>
       </c>
@@ -4334,10 +4336,10 @@
       <c r="V38" s="3"/>
     </row>
     <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="33">
+      <c r="A39" s="111">
         <v>37</v>
       </c>
-      <c r="B39" s="110"/>
+      <c r="B39" s="114"/>
       <c r="C39" s="70" t="s">
         <v>163</v>
       </c>
@@ -4402,21 +4404,21 @@
       <c r="I40" s="26"/>
       <c r="J40" s="26"/>
       <c r="K40" s="26"/>
-      <c r="L40" s="115" t="s">
+      <c r="L40" s="119" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="115"/>
-      <c r="N40" s="115"/>
-      <c r="O40" s="115"/>
+      <c r="M40" s="119"/>
+      <c r="N40" s="119"/>
+      <c r="O40" s="119"/>
       <c r="P40" s="30"/>
       <c r="Q40" s="30">
         <f>SUM(Q3:Q39)</f>
-        <v>205.65710000000001</v>
+        <v>199.66589999999999</v>
       </c>
       <c r="R40" s="30"/>
       <c r="S40" s="22">
         <f>SUM(S3:S39)</f>
-        <v>162.25650000000002</v>
+        <v>154.76600000000002</v>
       </c>
       <c r="T40" s="26"/>
       <c r="U40" s="3"/>
@@ -4427,24 +4429,24 @@
       <c r="I41" s="26"/>
       <c r="J41" s="28"/>
       <c r="K41" s="26"/>
-      <c r="L41" s="111" t="s">
+      <c r="L41" s="115" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="111"/>
-      <c r="N41" s="111"/>
-      <c r="O41" s="111"/>
+      <c r="M41" s="115"/>
+      <c r="N41" s="115"/>
+      <c r="O41" s="115"/>
       <c r="P41" s="22">
         <f>SUM(P3:P39)</f>
-        <v>32.938200000000002</v>
+        <v>31.930699999999991</v>
       </c>
       <c r="Q41" s="22">
         <f>Q40/5</f>
-        <v>41.131420000000006</v>
+        <v>39.93318</v>
       </c>
       <c r="R41" s="27"/>
       <c r="S41" s="29">
         <f>S40/5</f>
-        <v>32.451300000000003</v>
+        <v>30.953200000000002</v>
       </c>
       <c r="T41" s="26"/>
       <c r="U41" s="3"/>
@@ -4697,42 +4699,42 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="N4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="N5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="N6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="N7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="N10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="N14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="N16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="N17" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="N18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="N19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="N20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="N22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="N23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="N25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="N32" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="N33" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="N34" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="N36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="N37" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="N21" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="N39" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="N11" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="N13" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="N15" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="N35" r:id="rId36" xr:uid="{22803AA7-377B-442D-B7F9-22DAF87C6ADB}"/>
+    <hyperlink ref="N8" r:id="rId1"/>
+    <hyperlink ref="N3" r:id="rId2"/>
+    <hyperlink ref="N4" r:id="rId3"/>
+    <hyperlink ref="N5" r:id="rId4"/>
+    <hyperlink ref="N6" r:id="rId5"/>
+    <hyperlink ref="N7" r:id="rId6"/>
+    <hyperlink ref="N9" r:id="rId7"/>
+    <hyperlink ref="N10" r:id="rId8"/>
+    <hyperlink ref="N12" r:id="rId9"/>
+    <hyperlink ref="N14" r:id="rId10"/>
+    <hyperlink ref="N16" r:id="rId11"/>
+    <hyperlink ref="N17" r:id="rId12"/>
+    <hyperlink ref="N18" r:id="rId13"/>
+    <hyperlink ref="N19" r:id="rId14"/>
+    <hyperlink ref="N20" r:id="rId15"/>
+    <hyperlink ref="N22" r:id="rId16"/>
+    <hyperlink ref="N23" r:id="rId17"/>
+    <hyperlink ref="N24" r:id="rId18"/>
+    <hyperlink ref="N25" r:id="rId19"/>
+    <hyperlink ref="N26" r:id="rId20"/>
+    <hyperlink ref="N27" r:id="rId21"/>
+    <hyperlink ref="N28" r:id="rId22"/>
+    <hyperlink ref="N29" r:id="rId23"/>
+    <hyperlink ref="N30" r:id="rId24"/>
+    <hyperlink ref="N31" r:id="rId25"/>
+    <hyperlink ref="N32" r:id="rId26"/>
+    <hyperlink ref="N33" r:id="rId27"/>
+    <hyperlink ref="N34" r:id="rId28"/>
+    <hyperlink ref="N36" r:id="rId29"/>
+    <hyperlink ref="N37" r:id="rId30"/>
+    <hyperlink ref="N21" r:id="rId31"/>
+    <hyperlink ref="N39" r:id="rId32"/>
+    <hyperlink ref="N11" r:id="rId33"/>
+    <hyperlink ref="N13" r:id="rId34"/>
+    <hyperlink ref="N15" r:id="rId35"/>
+    <hyperlink ref="N35" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId37"/>

</xml_diff>

<commit_message>
LCSC and fabrication BOM reviewed.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SaleemD-CustomProduct\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDA3C3B-D461-4ED2-B074-3AE9D842EB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,7 +18,7 @@
   <definedNames>
     <definedName name="LCSC">Sheet1!$N$20</definedName>
   </definedNames>
-  <calcPr calcId="162913" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="246">
   <si>
     <t>S. No.</t>
   </si>
@@ -681,9 +682,6 @@
     <t>C381097</t>
   </si>
   <si>
-    <t>C255767</t>
-  </si>
-  <si>
     <t>C521664</t>
   </si>
   <si>
@@ -767,12 +765,27 @@
   </si>
   <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>SOFNG</t>
+  </si>
+  <si>
+    <t>C55208</t>
+  </si>
+  <si>
+    <t>X1A000061000200</t>
+  </si>
+  <si>
+    <t>Alternate has same footprint and manufacturer</t>
+  </si>
+  <si>
+    <t>Out of stock on LCSC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -894,7 +907,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -919,6 +932,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="28">
     <border>
@@ -1278,7 +1297,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1306,9 +1325,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1491,9 +1507,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1558,9 +1571,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="21" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1626,6 +1636,66 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1907,12 +1977,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="21" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" style="20" customWidth="1"/>
     <col min="3" max="3" width="47.5703125" customWidth="1"/>
     <col min="4" max="4" width="36.42578125" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
@@ -1933,486 +2003,486 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="116" t="s">
-        <v>240</v>
-      </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="118"/>
+      <c r="A1" s="113" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
+      <c r="H1" s="114"/>
+      <c r="I1" s="114"/>
+      <c r="J1" s="114"/>
+      <c r="K1" s="114"/>
+      <c r="L1" s="114"/>
+      <c r="M1" s="114"/>
+      <c r="N1" s="114"/>
+      <c r="O1" s="114"/>
+      <c r="P1" s="114"/>
+      <c r="Q1" s="114"/>
+      <c r="R1" s="114"/>
+      <c r="S1" s="114"/>
+      <c r="T1" s="115"/>
     </row>
     <row r="2" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="35" t="s">
+      <c r="F2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="35" t="s">
+      <c r="G2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="35" t="s">
+      <c r="H2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="35" t="s">
+      <c r="I2" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="35" t="s">
+      <c r="J2" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="35" t="s">
+      <c r="K2" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="35" t="s">
+      <c r="L2" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="35" t="s">
+      <c r="M2" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="36" t="s">
+      <c r="N2" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="31" t="s">
+      <c r="O2" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="31" t="s">
+      <c r="P2" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="31" t="s">
+      <c r="Q2" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="R2" s="31" t="s">
+      <c r="R2" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="32" t="s">
+      <c r="S2" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="35" t="s">
+      <c r="T2" s="34" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33">
+      <c r="A3" s="32">
         <v>1</v>
       </c>
-      <c r="B3" s="112" t="s">
+      <c r="B3" s="109" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="102" t="s">
+      <c r="D3" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="49" t="s">
         <v>192</v>
       </c>
-      <c r="I3" s="47" t="s">
+      <c r="I3" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="K3" s="52">
+      <c r="K3" s="51">
         <v>10</v>
       </c>
-      <c r="L3" s="67">
+      <c r="L3" s="66">
         <v>1</v>
       </c>
-      <c r="M3" s="52">
+      <c r="M3" s="51">
         <f>L3*5</f>
         <v>5</v>
       </c>
-      <c r="N3" s="53" t="s">
+      <c r="N3" s="52" t="s">
         <v>189</v>
       </c>
-      <c r="O3" s="54">
+      <c r="O3" s="53">
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="P3" s="55">
+      <c r="P3" s="54">
         <f>O3*L3</f>
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="Q3" s="55">
+      <c r="Q3" s="54">
         <f>O3*K3</f>
         <v>0.60899999999999999</v>
       </c>
-      <c r="R3" s="54">
+      <c r="R3" s="53">
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="S3" s="55">
+      <c r="S3" s="54">
         <f>R3*M3</f>
         <v>0.30449999999999999</v>
       </c>
-      <c r="T3" s="56"/>
+      <c r="T3" s="55"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
     </row>
     <row r="4" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33">
+      <c r="A4" s="32">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="18" t="s">
+      <c r="B4" s="110"/>
+      <c r="C4" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="100" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="16" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H4" s="37" t="s">
+      <c r="H4" s="36" t="s">
         <v>193</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="I4" s="36" t="s">
         <v>175</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="K4" s="39">
+      <c r="K4" s="38">
         <v>7</v>
       </c>
-      <c r="L4" s="15">
+      <c r="L4" s="14">
         <v>1</v>
       </c>
-      <c r="M4" s="39">
+      <c r="M4" s="38">
         <f t="shared" ref="M4:M39" si="0">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="57" t="s">
+      <c r="N4" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O4" s="40">
+      <c r="O4" s="39">
         <v>0.55730000000000002</v>
       </c>
-      <c r="P4" s="41">
+      <c r="P4" s="40">
         <f t="shared" ref="P4:P39" si="1">O4*L4</f>
         <v>0.55730000000000002</v>
       </c>
-      <c r="Q4" s="41">
+      <c r="Q4" s="40">
         <f t="shared" ref="Q4:Q39" si="2">O4*K4</f>
         <v>3.9011</v>
       </c>
-      <c r="R4" s="58">
+      <c r="R4" s="57">
         <v>0.55730000000000002</v>
       </c>
-      <c r="S4" s="41">
+      <c r="S4" s="40">
         <f t="shared" ref="S4:S39" si="3">R4*M4</f>
         <v>2.7865000000000002</v>
       </c>
-      <c r="T4" s="49"/>
+      <c r="T4" s="48"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
     </row>
     <row r="5" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33">
+      <c r="A5" s="32">
         <v>3</v>
       </c>
-      <c r="B5" s="113"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="110"/>
+      <c r="C5" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="103" t="s">
+      <c r="D5" s="100" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>41</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H5" s="37" t="s">
+      <c r="H5" s="36" t="s">
         <v>194</v>
       </c>
-      <c r="I5" s="38" t="s">
+      <c r="I5" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="J5" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="K5" s="39">
+      <c r="K5" s="38">
         <v>50</v>
       </c>
-      <c r="L5" s="15">
+      <c r="L5" s="14">
         <v>1</v>
       </c>
-      <c r="M5" s="39">
+      <c r="M5" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N5" s="57" t="s">
+      <c r="N5" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O5" s="40">
+      <c r="O5" s="39">
         <v>6.1000000000000004E-3</v>
       </c>
-      <c r="P5" s="41">
+      <c r="P5" s="40">
         <f t="shared" si="1"/>
         <v>6.1000000000000004E-3</v>
       </c>
-      <c r="Q5" s="41">
+      <c r="Q5" s="40">
         <f t="shared" si="2"/>
         <v>0.30499999999999999</v>
       </c>
-      <c r="R5" s="40">
+      <c r="R5" s="39">
         <v>6.1000000000000004E-3</v>
       </c>
-      <c r="S5" s="41">
+      <c r="S5" s="40">
         <f t="shared" si="3"/>
         <v>3.0500000000000003E-2</v>
       </c>
-      <c r="T5" s="49"/>
+      <c r="T5" s="48"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
     </row>
     <row r="6" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33">
+      <c r="A6" s="32">
         <v>4</v>
       </c>
-      <c r="B6" s="113"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="110"/>
+      <c r="C6" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="103" t="s">
+      <c r="D6" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="16" t="s">
         <v>45</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="36" t="s">
         <v>195</v>
       </c>
-      <c r="I6" s="38" t="s">
+      <c r="I6" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="J6" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="K6" s="39">
+      <c r="K6" s="38">
         <v>100</v>
       </c>
-      <c r="L6" s="15">
+      <c r="L6" s="14">
         <v>2</v>
       </c>
-      <c r="M6" s="39">
+      <c r="M6" s="38">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N6" s="59" t="s">
+      <c r="N6" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O6" s="66">
+      <c r="O6" s="65">
         <v>2.8E-3</v>
       </c>
-      <c r="P6" s="41">
+      <c r="P6" s="40">
         <f t="shared" si="1"/>
         <v>5.5999999999999999E-3</v>
       </c>
-      <c r="Q6" s="41">
+      <c r="Q6" s="40">
         <f t="shared" si="2"/>
         <v>0.27999999999999997</v>
       </c>
-      <c r="R6" s="66">
+      <c r="R6" s="65">
         <v>2.8E-3</v>
       </c>
-      <c r="S6" s="41">
+      <c r="S6" s="40">
         <f t="shared" si="3"/>
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="T6" s="49"/>
+      <c r="T6" s="48"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
     </row>
     <row r="7" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33">
+      <c r="A7" s="32">
         <v>5</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="110"/>
+      <c r="C7" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="103" t="s">
+      <c r="D7" s="100" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="64" t="s">
+      <c r="G7" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="37" t="s">
+      <c r="H7" s="36" t="s">
         <v>196</v>
       </c>
-      <c r="I7" s="38" t="s">
+      <c r="I7" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="K7" s="39">
+      <c r="K7" s="38">
         <v>100</v>
       </c>
-      <c r="L7" s="15">
+      <c r="L7" s="14">
         <v>14</v>
       </c>
-      <c r="M7" s="39">
+      <c r="M7" s="38">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="N7" s="59" t="s">
+      <c r="N7" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O7" s="40">
+      <c r="O7" s="39">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="P7" s="41">
+      <c r="P7" s="40">
         <f t="shared" si="1"/>
         <v>0.11480000000000001</v>
       </c>
-      <c r="Q7" s="41">
+      <c r="Q7" s="40">
         <f t="shared" si="2"/>
         <v>0.82000000000000006</v>
       </c>
-      <c r="R7" s="40">
+      <c r="R7" s="39">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="S7" s="41">
+      <c r="S7" s="40">
         <f t="shared" si="3"/>
         <v>0.57400000000000007</v>
       </c>
-      <c r="T7" s="19"/>
+      <c r="T7" s="18"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33">
+      <c r="A8" s="32">
         <v>6</v>
       </c>
-      <c r="B8" s="113"/>
-      <c r="C8" s="18" t="s">
+      <c r="B8" s="110"/>
+      <c r="C8" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="103" t="s">
+      <c r="D8" s="100" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="16" t="s">
         <v>52</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="37" t="s">
+      <c r="H8" s="36" t="s">
         <v>197</v>
       </c>
-      <c r="I8" s="38" t="s">
+      <c r="I8" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="K8" s="39">
+      <c r="K8" s="38">
         <v>20</v>
       </c>
-      <c r="L8" s="15">
+      <c r="L8" s="14">
         <v>2</v>
       </c>
-      <c r="M8" s="39">
+      <c r="M8" s="38">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="N8" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="O8" s="40">
+      <c r="O8" s="39">
         <v>2.98E-2</v>
       </c>
-      <c r="P8" s="41">
+      <c r="P8" s="40">
         <f t="shared" si="1"/>
         <v>5.96E-2</v>
       </c>
-      <c r="Q8" s="41">
+      <c r="Q8" s="40">
         <f t="shared" si="2"/>
         <v>0.59599999999999997</v>
       </c>
-      <c r="R8" s="40">
+      <c r="R8" s="39">
         <v>2.98E-2</v>
       </c>
-      <c r="S8" s="41">
+      <c r="S8" s="40">
         <f t="shared" si="3"/>
         <v>0.29799999999999999</v>
       </c>
-      <c r="T8" s="49"/>
+      <c r="T8" s="48"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33">
+      <c r="A9" s="32">
         <v>7</v>
       </c>
-      <c r="B9" s="113"/>
-      <c r="C9" s="16" t="s">
+      <c r="B9" s="110"/>
+      <c r="C9" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="37" t="s">
         <v>55</v>
       </c>
       <c r="E9" s="6" t="s">
@@ -2424,521 +2494,521 @@
       <c r="G9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="36" t="s">
         <v>198</v>
       </c>
-      <c r="I9" s="37" t="s">
+      <c r="I9" s="36" t="s">
         <v>175</v>
       </c>
-      <c r="J9" s="17" t="s">
+      <c r="J9" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="K9" s="39">
+      <c r="K9" s="38">
         <v>50</v>
       </c>
-      <c r="L9" s="15">
+      <c r="L9" s="14">
         <v>7</v>
       </c>
-      <c r="M9" s="39">
+      <c r="M9" s="38">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="N9" s="59" t="s">
+      <c r="N9" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O9" s="58">
-        <v>1.0200000000000001E-2</v>
-      </c>
-      <c r="P9" s="41">
-        <f t="shared" si="1"/>
-        <v>7.1400000000000005E-2</v>
-      </c>
-      <c r="Q9" s="41">
+      <c r="O9" s="57">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="P9" s="40">
+        <f>O9*L9</f>
+        <v>5.1799999999999999E-2</v>
+      </c>
+      <c r="Q9" s="40">
         <f t="shared" si="2"/>
-        <v>0.51</v>
-      </c>
-      <c r="R9" s="58">
-        <v>1.0200000000000001E-2</v>
-      </c>
-      <c r="S9" s="41">
+        <v>0.37</v>
+      </c>
+      <c r="R9" s="57">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="S9" s="40">
         <f t="shared" si="3"/>
-        <v>0.35700000000000004</v>
-      </c>
-      <c r="T9" s="49"/>
+        <v>0.25900000000000001</v>
+      </c>
+      <c r="T9" s="48"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33">
+      <c r="A10" s="32">
         <v>8</v>
       </c>
-      <c r="B10" s="113"/>
-      <c r="C10" s="18" t="s">
+      <c r="B10" s="110"/>
+      <c r="C10" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="103" t="s">
+      <c r="D10" s="100" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="100" t="s">
+      <c r="F10" s="97" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="64" t="s">
+      <c r="G10" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="37" t="s">
+      <c r="H10" s="36" t="s">
         <v>199</v>
       </c>
-      <c r="I10" s="39" t="s">
+      <c r="I10" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="J10" s="17" t="s">
+      <c r="J10" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="K10" s="39">
+      <c r="K10" s="38">
         <v>20</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="14">
         <v>2</v>
       </c>
-      <c r="M10" s="39">
+      <c r="M10" s="38">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N10" s="59" t="s">
+      <c r="N10" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O10" s="40">
+      <c r="O10" s="39">
         <v>3.5400000000000001E-2</v>
       </c>
-      <c r="P10" s="41">
+      <c r="P10" s="40">
         <f t="shared" si="1"/>
         <v>7.0800000000000002E-2</v>
       </c>
-      <c r="Q10" s="41">
+      <c r="Q10" s="40">
         <f t="shared" si="2"/>
         <v>0.70799999999999996</v>
       </c>
-      <c r="R10" s="58">
+      <c r="R10" s="57">
         <v>3.5400000000000001E-2</v>
       </c>
-      <c r="S10" s="41">
+      <c r="S10" s="40">
         <f t="shared" si="3"/>
         <v>0.35399999999999998</v>
       </c>
-      <c r="T10" s="19"/>
+      <c r="T10" s="18"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33">
+      <c r="A11" s="32">
         <v>9</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="18" t="s">
+      <c r="B11" s="110"/>
+      <c r="C11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="103" t="s">
+      <c r="D11" s="100" t="s">
         <v>62</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="101" t="s">
+      <c r="F11" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="64" t="s">
+      <c r="G11" s="63" t="s">
+        <v>226</v>
+      </c>
+      <c r="H11" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="I11" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="H11" s="37" t="s">
-        <v>232</v>
-      </c>
-      <c r="I11" s="39" t="s">
-        <v>228</v>
-      </c>
-      <c r="J11" s="17" t="s">
+      <c r="J11" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="K11" s="39">
+      <c r="K11" s="38">
         <v>100</v>
       </c>
-      <c r="L11" s="15">
+      <c r="L11" s="14">
         <v>2</v>
       </c>
-      <c r="M11" s="39">
+      <c r="M11" s="38">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N11" s="96" t="s">
+      <c r="N11" s="94" t="s">
         <v>189</v>
       </c>
-      <c r="O11" s="40">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="P11" s="41">
+      <c r="O11" s="39">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="P11" s="40">
         <f t="shared" si="1"/>
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="Q11" s="40">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="Q11" s="39">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="R11" s="40">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="S11" s="41">
+      <c r="R11" s="39">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="S11" s="40">
         <f t="shared" si="3"/>
-        <v>0.03</v>
-      </c>
-      <c r="T11" s="19"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="T11" s="18"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="33">
+      <c r="A12" s="32">
         <v>10</v>
       </c>
-      <c r="B12" s="114"/>
-      <c r="C12" s="70" t="s">
+      <c r="B12" s="111"/>
+      <c r="C12" s="69" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="104" t="s">
+      <c r="D12" s="101" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="68" t="s">
+      <c r="E12" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="68" t="s">
+      <c r="F12" s="67" t="s">
         <v>66</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="60" t="s">
+      <c r="H12" s="59" t="s">
         <v>200</v>
       </c>
-      <c r="I12" s="46" t="s">
+      <c r="I12" s="45" t="s">
         <v>175</v>
       </c>
-      <c r="J12" s="68" t="s">
+      <c r="J12" s="67" t="s">
         <v>174</v>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="44">
         <v>50</v>
       </c>
-      <c r="L12" s="69">
+      <c r="L12" s="68">
         <v>2</v>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="44">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N12" s="61" t="s">
+      <c r="N12" s="60" t="s">
         <v>189</v>
       </c>
-      <c r="O12" s="42">
+      <c r="O12" s="41">
         <v>5.1000000000000004E-3</v>
       </c>
-      <c r="P12" s="43">
+      <c r="P12" s="42">
         <f t="shared" si="1"/>
         <v>1.0200000000000001E-2</v>
       </c>
-      <c r="Q12" s="43">
+      <c r="Q12" s="42">
         <f t="shared" si="2"/>
         <v>0.255</v>
       </c>
-      <c r="R12" s="42">
+      <c r="R12" s="41">
         <v>5.1000000000000004E-3</v>
       </c>
-      <c r="S12" s="43">
+      <c r="S12" s="42">
         <f t="shared" si="3"/>
         <v>5.1000000000000004E-2</v>
       </c>
-      <c r="T12" s="62"/>
+      <c r="T12" s="61"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="33">
+      <c r="A13" s="32">
         <v>11</v>
       </c>
-      <c r="B13" s="112" t="s">
+      <c r="B13" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="102" t="s">
+      <c r="D13" s="99" t="s">
         <v>69</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="99" t="s">
+      <c r="F13" s="96" t="s">
         <v>71</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H13" s="50" t="s">
-        <v>231</v>
-      </c>
-      <c r="I13" s="48" t="s">
-        <v>229</v>
+      <c r="H13" s="49" t="s">
+        <v>230</v>
+      </c>
+      <c r="I13" s="47" t="s">
+        <v>228</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="K13" s="52">
+      <c r="K13" s="51">
         <v>40</v>
       </c>
-      <c r="L13" s="67">
+      <c r="L13" s="66">
         <v>4</v>
       </c>
-      <c r="M13" s="52">
+      <c r="M13" s="51">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N13" s="71" t="s">
+      <c r="N13" s="70" t="s">
         <v>189</v>
       </c>
-      <c r="O13" s="54">
+      <c r="O13" s="53">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="P13" s="55">
+      <c r="P13" s="54">
         <f t="shared" si="1"/>
         <v>6.9599999999999995E-2</v>
       </c>
-      <c r="Q13" s="55">
+      <c r="Q13" s="54">
         <f t="shared" si="2"/>
         <v>0.69599999999999995</v>
       </c>
-      <c r="R13" s="54">
+      <c r="R13" s="53">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="S13" s="55">
+      <c r="S13" s="54">
         <f t="shared" si="3"/>
         <v>0.34799999999999998</v>
       </c>
-      <c r="T13" s="12"/>
+      <c r="T13" s="11"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33">
+      <c r="A14" s="32">
         <v>12</v>
       </c>
-      <c r="B14" s="114"/>
-      <c r="C14" s="73" t="s">
+      <c r="B14" s="111"/>
+      <c r="C14" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="104" t="s">
+      <c r="D14" s="101" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="68" t="s">
+      <c r="E14" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="F14" s="68" t="s">
+      <c r="F14" s="67" t="s">
         <v>76</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="H14" s="60" t="s">
+      <c r="H14" s="59" t="s">
         <v>201</v>
       </c>
-      <c r="I14" s="46" t="s">
+      <c r="I14" s="45" t="s">
         <v>175</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="K14" s="45">
+      <c r="K14" s="44">
         <v>12</v>
       </c>
-      <c r="L14" s="69">
+      <c r="L14" s="68">
         <v>2</v>
       </c>
-      <c r="M14" s="45">
+      <c r="M14" s="44">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N14" s="61" t="s">
+      <c r="N14" s="60" t="s">
         <v>189</v>
       </c>
-      <c r="O14" s="42">
+      <c r="O14" s="41">
         <v>0.93589999999999995</v>
       </c>
-      <c r="P14" s="43">
+      <c r="P14" s="42">
         <f t="shared" si="1"/>
         <v>1.8717999999999999</v>
       </c>
-      <c r="Q14" s="43">
+      <c r="Q14" s="42">
         <f t="shared" si="2"/>
         <v>11.230799999999999</v>
       </c>
-      <c r="R14" s="42">
+      <c r="R14" s="41">
         <v>0.69069999999999998</v>
       </c>
-      <c r="S14" s="43">
+      <c r="S14" s="42">
         <f t="shared" si="3"/>
         <v>6.907</v>
       </c>
-      <c r="T14" s="62"/>
+      <c r="T14" s="61"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33">
+      <c r="A15" s="32">
         <v>13</v>
       </c>
-      <c r="B15" s="110" t="s">
+      <c r="B15" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="76" t="s">
+      <c r="C15" s="74" t="s">
+        <v>234</v>
+      </c>
+      <c r="D15" s="102" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="75" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" s="75" t="s">
         <v>235</v>
       </c>
-      <c r="D15" s="105" t="s">
-        <v>78</v>
-      </c>
-      <c r="E15" s="77" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="77" t="s">
+      <c r="G15" s="76" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="77" t="s">
         <v>236</v>
       </c>
-      <c r="G15" s="78" t="s">
-        <v>79</v>
-      </c>
-      <c r="H15" s="79" t="s">
-        <v>237</v>
-      </c>
-      <c r="I15" s="80"/>
-      <c r="J15" s="77" t="s">
+      <c r="I15" s="78"/>
+      <c r="J15" s="75" t="s">
         <v>176</v>
       </c>
-      <c r="K15" s="81">
+      <c r="K15" s="79">
         <v>7</v>
       </c>
-      <c r="L15" s="82">
+      <c r="L15" s="80">
         <v>1</v>
       </c>
-      <c r="M15" s="81">
+      <c r="M15" s="79">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N15" s="98" t="s">
+      <c r="N15" s="95" t="s">
         <v>189</v>
       </c>
-      <c r="O15" s="83">
+      <c r="O15" s="81">
         <v>0.87980000000000003</v>
       </c>
-      <c r="P15" s="84">
+      <c r="P15" s="82">
         <f t="shared" si="1"/>
         <v>0.87980000000000003</v>
       </c>
-      <c r="Q15" s="84">
+      <c r="Q15" s="82">
         <f t="shared" si="2"/>
         <v>6.1585999999999999</v>
       </c>
-      <c r="R15" s="83">
+      <c r="R15" s="81">
         <v>0.87980000000000003</v>
       </c>
-      <c r="S15" s="84">
+      <c r="S15" s="82">
         <f t="shared" si="3"/>
         <v>4.399</v>
       </c>
-      <c r="T15" s="95"/>
+      <c r="T15" s="93"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
     </row>
     <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33">
+      <c r="A16" s="32">
         <v>14</v>
       </c>
-      <c r="B16" s="85" t="s">
+      <c r="B16" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="86" t="s">
+      <c r="C16" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="106" t="s">
+      <c r="D16" s="103" t="s">
         <v>81</v>
       </c>
-      <c r="E16" s="87" t="s">
+      <c r="E16" s="85" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="87" t="s">
+      <c r="F16" s="85" t="s">
         <v>83</v>
       </c>
-      <c r="G16" s="87" t="s">
+      <c r="G16" s="85" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="88" t="s">
+      <c r="H16" s="86" t="s">
         <v>202</v>
       </c>
-      <c r="I16" s="89" t="s">
+      <c r="I16" s="87" t="s">
         <v>175</v>
       </c>
-      <c r="J16" s="87" t="s">
+      <c r="J16" s="85" t="s">
         <v>175</v>
       </c>
-      <c r="K16" s="63">
+      <c r="K16" s="62">
         <v>20</v>
       </c>
-      <c r="L16" s="90">
+      <c r="L16" s="88">
         <v>1</v>
       </c>
-      <c r="M16" s="63">
+      <c r="M16" s="62">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N16" s="91" t="s">
+      <c r="N16" s="89" t="s">
         <v>189</v>
       </c>
-      <c r="O16" s="92">
+      <c r="O16" s="90">
         <v>4.07E-2</v>
       </c>
-      <c r="P16" s="93">
+      <c r="P16" s="91">
         <f t="shared" si="1"/>
         <v>4.07E-2</v>
       </c>
-      <c r="Q16" s="93">
+      <c r="Q16" s="91">
         <f t="shared" si="2"/>
         <v>0.81400000000000006</v>
       </c>
-      <c r="R16" s="92">
+      <c r="R16" s="90">
         <v>4.07E-2</v>
       </c>
-      <c r="S16" s="93">
+      <c r="S16" s="91">
         <f t="shared" si="3"/>
         <v>0.20350000000000001</v>
       </c>
-      <c r="T16" s="94"/>
+      <c r="T16" s="92"/>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
     </row>
     <row r="17" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33">
+      <c r="A17" s="32">
         <v>15</v>
       </c>
-      <c r="B17" s="112" t="s">
+      <c r="B17" s="109" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="102" t="s">
+      <c r="D17" s="99" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E17" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="G17" s="14" t="s">
+      <c r="G17" s="13" t="s">
         <v>89</v>
       </c>
       <c r="H17" s="1" t="s">
@@ -2947,628 +3017,630 @@
       <c r="I17" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J17" s="14" t="s">
+      <c r="J17" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="K17" s="52">
+      <c r="K17" s="51">
         <v>50</v>
       </c>
-      <c r="L17" s="67">
+      <c r="L17" s="66">
         <v>1</v>
       </c>
-      <c r="M17" s="52">
+      <c r="M17" s="51">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N17" s="71" t="s">
+      <c r="N17" s="70" t="s">
         <v>189</v>
       </c>
-      <c r="O17" s="54">
+      <c r="O17" s="53">
         <v>1.8E-3</v>
       </c>
-      <c r="P17" s="55">
+      <c r="P17" s="54">
         <f t="shared" si="1"/>
         <v>1.8E-3</v>
       </c>
-      <c r="Q17" s="55">
+      <c r="Q17" s="54">
         <f t="shared" si="2"/>
         <v>0.09</v>
       </c>
-      <c r="R17" s="54">
+      <c r="R17" s="53">
         <v>1.8E-3</v>
       </c>
-      <c r="S17" s="55">
+      <c r="S17" s="54">
         <f t="shared" si="3"/>
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="T17" s="72"/>
+      <c r="T17" s="71"/>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
     </row>
     <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="33">
+      <c r="A18" s="32">
         <v>16</v>
       </c>
-      <c r="B18" s="113"/>
-      <c r="C18" s="18" t="s">
+      <c r="B18" s="110"/>
+      <c r="C18" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="103" t="s">
+      <c r="D18" s="100" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="16" t="s">
         <v>92</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="51" t="s">
+      <c r="H18" s="50" t="s">
         <v>204</v>
       </c>
-      <c r="I18" s="39" t="s">
+      <c r="I18" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="J18" s="17" t="s">
+      <c r="J18" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="K18" s="39">
+      <c r="K18" s="38">
         <v>10</v>
       </c>
-      <c r="L18" s="15">
+      <c r="L18" s="14">
         <v>1</v>
       </c>
-      <c r="M18" s="39">
+      <c r="M18" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N18" s="59" t="s">
+      <c r="N18" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O18" s="40">
+      <c r="O18" s="39">
         <v>6.0699999999999997E-2</v>
       </c>
-      <c r="P18" s="41">
+      <c r="P18" s="40">
         <f t="shared" si="1"/>
         <v>6.0699999999999997E-2</v>
       </c>
-      <c r="Q18" s="41">
+      <c r="Q18" s="40">
         <f t="shared" si="2"/>
         <v>0.60699999999999998</v>
       </c>
-      <c r="R18" s="40">
+      <c r="R18" s="39">
         <v>6.0699999999999997E-2</v>
       </c>
-      <c r="S18" s="41">
+      <c r="S18" s="40">
         <f t="shared" si="3"/>
         <v>0.30349999999999999</v>
       </c>
-      <c r="T18" s="20"/>
+      <c r="T18" s="19"/>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
     </row>
     <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33">
+      <c r="A19" s="32">
         <v>17</v>
       </c>
-      <c r="B19" s="113"/>
-      <c r="C19" s="18" t="s">
+      <c r="B19" s="110"/>
+      <c r="C19" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="103" t="s">
+      <c r="D19" s="100" t="s">
         <v>95</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="16" t="s">
         <v>96</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H19" s="39" t="s">
+      <c r="H19" s="38" t="s">
         <v>205</v>
       </c>
-      <c r="I19" s="51" t="s">
+      <c r="I19" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="J19" s="17" t="s">
+      <c r="J19" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="K19" s="39">
+      <c r="K19" s="38">
         <v>100</v>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="14">
         <v>1</v>
       </c>
-      <c r="M19" s="39">
+      <c r="M19" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="59" t="s">
+      <c r="N19" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O19" s="40">
+      <c r="O19" s="39">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="P19" s="41">
+      <c r="P19" s="40">
         <f t="shared" si="1"/>
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="Q19" s="41">
+      <c r="Q19" s="40">
         <f t="shared" si="2"/>
         <v>0.24</v>
       </c>
-      <c r="R19" s="40">
+      <c r="R19" s="39">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="S19" s="41">
+      <c r="S19" s="40">
         <f t="shared" si="3"/>
         <v>1.1999999999999999E-2</v>
       </c>
-      <c r="T19" s="49"/>
+      <c r="T19" s="48"/>
       <c r="U19" s="3"/>
       <c r="V19" s="3"/>
     </row>
     <row r="20" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="33">
+      <c r="A20" s="32">
         <v>18</v>
       </c>
-      <c r="B20" s="113"/>
-      <c r="C20" s="18" t="s">
+      <c r="B20" s="110"/>
+      <c r="C20" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="103" t="s">
+      <c r="D20" s="100" t="s">
         <v>98</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="16" t="s">
         <v>99</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H20" s="37" t="s">
+      <c r="H20" s="36" t="s">
         <v>206</v>
       </c>
-      <c r="I20" s="51" t="s">
+      <c r="I20" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="J20" s="17" t="s">
+      <c r="J20" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="K20" s="39">
+      <c r="K20" s="38">
         <v>100</v>
       </c>
-      <c r="L20" s="15">
+      <c r="L20" s="14">
         <v>6</v>
       </c>
-      <c r="M20" s="39">
+      <c r="M20" s="38">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N20" s="57" t="s">
+      <c r="N20" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O20" s="40">
+      <c r="O20" s="39">
         <v>1.4E-3</v>
       </c>
-      <c r="P20" s="41">
+      <c r="P20" s="40">
         <f t="shared" si="1"/>
         <v>8.3999999999999995E-3</v>
       </c>
-      <c r="Q20" s="41">
+      <c r="Q20" s="40">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
-      <c r="R20" s="40">
+      <c r="R20" s="39">
         <v>1.4E-3</v>
       </c>
-      <c r="S20" s="41">
+      <c r="S20" s="40">
         <f t="shared" si="3"/>
         <v>4.2000000000000003E-2</v>
       </c>
-      <c r="T20" s="49"/>
+      <c r="T20" s="48"/>
       <c r="U20" s="3"/>
       <c r="V20" s="3"/>
     </row>
     <row r="21" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33">
+      <c r="A21" s="32">
         <v>19</v>
       </c>
-      <c r="B21" s="113"/>
-      <c r="C21" s="16" t="s">
+      <c r="B21" s="110"/>
+      <c r="C21" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="D21" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="D21" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>239</v>
-      </c>
       <c r="F21" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H21" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="G21" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="H21" s="37" t="s">
-        <v>224</v>
-      </c>
-      <c r="I21" s="37" t="s">
+      <c r="I21" s="36" t="s">
         <v>175</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="J21" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="K21" s="39">
+      <c r="K21" s="38">
         <v>40</v>
       </c>
-      <c r="L21" s="15">
+      <c r="L21" s="14">
         <v>4</v>
       </c>
-      <c r="M21" s="39">
+      <c r="M21" s="38">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N21" s="57" t="s">
+      <c r="N21" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O21" s="40">
+      <c r="O21" s="39">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="P21" s="41">
+      <c r="P21" s="40">
         <f t="shared" si="1"/>
         <v>0.15040000000000001</v>
       </c>
-      <c r="Q21" s="41">
+      <c r="Q21" s="40">
         <f t="shared" si="2"/>
         <v>1.504</v>
       </c>
-      <c r="R21" s="40">
+      <c r="R21" s="39">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="S21" s="41">
+      <c r="S21" s="40">
         <f t="shared" si="3"/>
         <v>0.752</v>
       </c>
-      <c r="T21" s="49"/>
+      <c r="T21" s="48"/>
       <c r="U21" s="3"/>
       <c r="V21" s="3"/>
     </row>
     <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33">
+      <c r="A22" s="32">
         <v>20</v>
       </c>
-      <c r="B22" s="113"/>
-      <c r="C22" s="18" t="s">
+      <c r="B22" s="110"/>
+      <c r="C22" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="103" t="s">
+      <c r="D22" s="100" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="16" t="s">
         <v>103</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H22" s="37" t="s">
+      <c r="H22" s="36" t="s">
         <v>207</v>
       </c>
-      <c r="I22" s="51" t="s">
+      <c r="I22" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="J22" s="17" t="s">
+      <c r="J22" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="K22" s="39">
+      <c r="K22" s="38">
         <v>100</v>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="14">
         <v>4</v>
       </c>
-      <c r="M22" s="39">
+      <c r="M22" s="38">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N22" s="57" t="s">
+      <c r="N22" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O22" s="40">
+      <c r="O22" s="39">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="P22" s="41">
+      <c r="P22" s="40">
         <f t="shared" si="1"/>
         <v>6.7999999999999996E-3</v>
       </c>
-      <c r="Q22" s="41">
+      <c r="Q22" s="40">
         <f t="shared" si="2"/>
         <v>0.16999999999999998</v>
       </c>
-      <c r="R22" s="40">
+      <c r="R22" s="39">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="S22" s="41">
+      <c r="S22" s="40">
         <f t="shared" si="3"/>
         <v>3.3999999999999996E-2</v>
       </c>
-      <c r="T22" s="49"/>
+      <c r="T22" s="48"/>
       <c r="U22" s="3"/>
       <c r="V22" s="3"/>
     </row>
     <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="33">
+      <c r="A23" s="32">
         <v>21</v>
       </c>
-      <c r="B23" s="113"/>
-      <c r="C23" s="18" t="s">
+      <c r="B23" s="110"/>
+      <c r="C23" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="103" t="s">
+      <c r="D23" s="100" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="16" t="s">
         <v>106</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H23" s="37" t="s">
+      <c r="H23" s="36" t="s">
         <v>208</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J23" s="17" t="s">
+      <c r="J23" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="K23" s="39">
+      <c r="K23" s="38">
         <v>50</v>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="14">
         <v>4</v>
       </c>
-      <c r="M23" s="39">
+      <c r="M23" s="38">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N23" s="59" t="s">
+      <c r="N23" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O23" s="40">
+      <c r="O23" s="39">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="P23" s="41">
+      <c r="P23" s="40">
         <f t="shared" si="1"/>
         <v>0.06</v>
       </c>
-      <c r="Q23" s="41">
+      <c r="Q23" s="40">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-      <c r="R23" s="40">
+      <c r="R23" s="39">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="S23" s="41">
+      <c r="S23" s="40">
         <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
-      <c r="T23" s="49"/>
+      <c r="T23" s="48"/>
       <c r="U23" s="3"/>
       <c r="V23" s="3"/>
     </row>
     <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="33">
+      <c r="A24" s="32">
         <v>22</v>
       </c>
-      <c r="B24" s="113"/>
-      <c r="C24" s="18" t="s">
+      <c r="B24" s="110"/>
+      <c r="C24" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="D24" s="103" t="s">
+      <c r="D24" s="100" t="s">
         <v>108</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="16" t="s">
         <v>109</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="37" t="s">
+      <c r="H24" s="36" t="s">
         <v>209</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J24" s="17" t="s">
+      <c r="J24" s="16" t="s">
         <v>184</v>
       </c>
       <c r="K24" s="5">
         <v>100</v>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="14">
         <v>1</v>
       </c>
-      <c r="M24" s="39">
+      <c r="M24" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="59" t="s">
+      <c r="N24" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O24" s="40">
+      <c r="O24" s="39">
         <v>1.4E-3</v>
       </c>
-      <c r="P24" s="41">
+      <c r="P24" s="40">
         <f t="shared" si="1"/>
         <v>1.4E-3</v>
       </c>
-      <c r="Q24" s="41">
+      <c r="Q24" s="40">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
-      <c r="R24" s="40">
+      <c r="R24" s="39">
         <v>1.4E-3</v>
       </c>
-      <c r="S24" s="41">
+      <c r="S24" s="40">
         <f t="shared" si="3"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="T24" s="49"/>
+      <c r="T24" s="48"/>
       <c r="U24" s="3"/>
       <c r="V24" s="3"/>
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="33">
+      <c r="A25" s="32">
         <v>23</v>
       </c>
-      <c r="B25" s="114"/>
-      <c r="C25" s="70" t="s">
+      <c r="B25" s="111"/>
+      <c r="C25" s="69" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="104" t="s">
+      <c r="D25" s="101" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="68" t="s">
+      <c r="E25" s="67" t="s">
         <v>87</v>
       </c>
-      <c r="F25" s="68" t="s">
+      <c r="F25" s="67" t="s">
         <v>112</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="60" t="s">
+      <c r="H25" s="59" t="s">
         <v>210</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="J25" s="68" t="s">
+      <c r="J25" s="67" t="s">
         <v>185</v>
       </c>
       <c r="K25" s="8">
         <v>100</v>
       </c>
-      <c r="L25" s="69">
+      <c r="L25" s="68">
         <v>1</v>
       </c>
-      <c r="M25" s="45">
+      <c r="M25" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N25" s="61" t="s">
+      <c r="N25" s="60" t="s">
         <v>189</v>
       </c>
-      <c r="O25" s="42">
+      <c r="O25" s="41">
         <v>1.5E-3</v>
       </c>
-      <c r="P25" s="43">
+      <c r="P25" s="42">
         <f t="shared" si="1"/>
         <v>1.5E-3</v>
       </c>
-      <c r="Q25" s="43">
+      <c r="Q25" s="42">
         <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
-      <c r="R25" s="42">
+      <c r="R25" s="41">
         <v>1.5E-3</v>
       </c>
-      <c r="S25" s="43">
+      <c r="S25" s="42">
         <f t="shared" si="3"/>
         <v>7.4999999999999997E-3</v>
       </c>
-      <c r="T25" s="62"/>
+      <c r="T25" s="61"/>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
     </row>
     <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="33">
+      <c r="A26" s="32">
         <v>24</v>
       </c>
-      <c r="B26" s="112" t="s">
+      <c r="B26" s="109" t="s">
         <v>190</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="126" t="s">
         <v>113</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="118" t="s">
         <v>114</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="118" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="118" t="s">
         <v>115</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" s="119" t="s">
         <v>116</v>
       </c>
-      <c r="H26" s="50" t="s">
-        <v>230</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="H26" s="120" t="s">
+        <v>229</v>
+      </c>
+      <c r="I26" s="119" t="s">
         <v>175</v>
       </c>
-      <c r="J26" s="2" t="s">
+      <c r="J26" s="119" t="s">
         <v>175</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="119">
         <v>12</v>
       </c>
-      <c r="L26" s="67">
+      <c r="L26" s="122">
         <v>2</v>
       </c>
-      <c r="M26" s="52">
+      <c r="M26" s="123">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N26" s="97" t="s">
+      <c r="N26" s="127" t="s">
         <v>189</v>
       </c>
-      <c r="O26" s="54">
+      <c r="O26" s="124">
         <v>0.88370000000000004</v>
       </c>
-      <c r="P26" s="55">
+      <c r="P26" s="125">
         <f t="shared" si="1"/>
         <v>1.7674000000000001</v>
       </c>
-      <c r="Q26" s="55">
+      <c r="Q26" s="125">
         <f t="shared" si="2"/>
         <v>10.6044</v>
       </c>
-      <c r="R26" s="54">
+      <c r="R26" s="124">
         <v>0.65820000000000001</v>
       </c>
-      <c r="S26" s="55">
+      <c r="S26" s="125">
         <f t="shared" si="3"/>
         <v>6.5819999999999999</v>
       </c>
-      <c r="T26" s="56"/>
+      <c r="T26" s="55" t="s">
+        <v>245</v>
+      </c>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
     </row>
     <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="33">
+      <c r="A27" s="32">
         <v>25</v>
       </c>
-      <c r="B27" s="114"/>
-      <c r="C27" s="73" t="s">
+      <c r="B27" s="111"/>
+      <c r="C27" s="72" t="s">
         <v>117</v>
       </c>
       <c r="D27" s="10" t="s">
@@ -3583,7 +3655,7 @@
       <c r="G27" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H27" s="60" t="s">
+      <c r="H27" s="59" t="s">
         <v>212</v>
       </c>
       <c r="I27" s="8" t="s">
@@ -3595,126 +3667,128 @@
       <c r="K27" s="8">
         <v>7</v>
       </c>
-      <c r="L27" s="69">
+      <c r="L27" s="68">
         <v>1</v>
       </c>
-      <c r="M27" s="45">
+      <c r="M27" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="61" t="s">
+      <c r="N27" s="60" t="s">
         <v>189</v>
       </c>
-      <c r="O27" s="42">
+      <c r="O27" s="41">
         <v>0.28449999999999998</v>
       </c>
-      <c r="P27" s="43">
+      <c r="P27" s="42">
         <f t="shared" si="1"/>
         <v>0.28449999999999998</v>
       </c>
-      <c r="Q27" s="43">
+      <c r="Q27" s="42">
         <f t="shared" si="2"/>
         <v>1.9914999999999998</v>
       </c>
-      <c r="R27" s="42">
+      <c r="R27" s="41">
         <v>0.28449999999999998</v>
       </c>
-      <c r="S27" s="43">
+      <c r="S27" s="42">
         <f t="shared" si="3"/>
         <v>1.4224999999999999</v>
       </c>
-      <c r="T27" s="62"/>
+      <c r="T27" s="61"/>
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
     </row>
     <row r="28" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="33">
+      <c r="A28" s="32">
         <v>26</v>
       </c>
-      <c r="B28" s="112" t="s">
+      <c r="B28" s="109" t="s">
         <v>191</v>
       </c>
-      <c r="C28" s="74" t="s">
+      <c r="C28" s="117" t="s">
         <v>121</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="118" t="s">
         <v>122</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="118" t="s">
         <v>51</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="118" t="s">
         <v>123</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" s="119" t="s">
         <v>120</v>
       </c>
-      <c r="H28" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="J28" s="11" t="s">
+      <c r="H28" s="120" t="s">
+        <v>242</v>
+      </c>
+      <c r="I28" s="119" t="s">
+        <v>243</v>
+      </c>
+      <c r="J28" s="121" t="s">
         <v>186</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="119">
         <v>7</v>
       </c>
-      <c r="L28" s="67">
+      <c r="L28" s="122">
         <v>1</v>
       </c>
-      <c r="M28" s="52">
+      <c r="M28" s="123">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N28" s="71" t="s">
+      <c r="N28" s="127" t="s">
         <v>189</v>
       </c>
-      <c r="O28" s="54">
-        <v>0.49590000000000001</v>
-      </c>
-      <c r="P28" s="55">
+      <c r="O28" s="124">
+        <v>0.56630000000000003</v>
+      </c>
+      <c r="P28" s="125">
         <f t="shared" si="1"/>
-        <v>0.49590000000000001</v>
-      </c>
-      <c r="Q28" s="55">
+        <v>0.56630000000000003</v>
+      </c>
+      <c r="Q28" s="125">
         <f t="shared" si="2"/>
-        <v>3.4713000000000003</v>
-      </c>
-      <c r="R28" s="54">
-        <v>0.49590000000000001</v>
-      </c>
-      <c r="S28" s="55">
+        <v>3.9641000000000002</v>
+      </c>
+      <c r="R28" s="124">
+        <v>0.56630000000000003</v>
+      </c>
+      <c r="S28" s="125">
         <f t="shared" si="3"/>
-        <v>2.4794999999999998</v>
-      </c>
-      <c r="T28" s="56"/>
+        <v>2.8315000000000001</v>
+      </c>
+      <c r="T28" s="55" t="s">
+        <v>244</v>
+      </c>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
     </row>
     <row r="29" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="33">
+      <c r="A29" s="32">
         <v>27</v>
       </c>
-      <c r="B29" s="114"/>
-      <c r="C29" s="73" t="s">
+      <c r="B29" s="111"/>
+      <c r="C29" s="72" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="68" t="s">
+      <c r="D29" s="67" t="s">
         <v>125</v>
       </c>
-      <c r="E29" s="68" t="s">
+      <c r="E29" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="F29" s="68" t="s">
+      <c r="F29" s="67" t="s">
         <v>126</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="H29" s="60" t="s">
-        <v>214</v>
+      <c r="H29" s="59" t="s">
+        <v>213</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>175</v>
@@ -3725,64 +3799,64 @@
       <c r="K29" s="8">
         <v>7</v>
       </c>
-      <c r="L29" s="69">
+      <c r="L29" s="68">
         <v>1</v>
       </c>
-      <c r="M29" s="45">
+      <c r="M29" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N29" s="61" t="s">
+      <c r="N29" s="60" t="s">
         <v>189</v>
       </c>
-      <c r="O29" s="42">
+      <c r="O29" s="41">
         <v>0.41120000000000001</v>
       </c>
-      <c r="P29" s="43">
+      <c r="P29" s="42">
         <f t="shared" si="1"/>
         <v>0.41120000000000001</v>
       </c>
-      <c r="Q29" s="43">
+      <c r="Q29" s="42">
         <f t="shared" si="2"/>
         <v>2.8784000000000001</v>
       </c>
-      <c r="R29" s="42">
+      <c r="R29" s="41">
         <v>0.41120000000000001</v>
       </c>
-      <c r="S29" s="43">
+      <c r="S29" s="42">
         <f t="shared" si="3"/>
         <v>2.056</v>
       </c>
-      <c r="T29" s="62"/>
+      <c r="T29" s="61"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
     </row>
     <row r="30" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="33">
+      <c r="A30" s="32">
         <v>28</v>
       </c>
-      <c r="B30" s="112" t="s">
+      <c r="B30" s="109" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="F30" s="13" t="s">
         <v>131</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="H30" s="50" t="s">
-        <v>215</v>
-      </c>
-      <c r="I30" s="50" t="s">
+      <c r="H30" s="49" t="s">
+        <v>214</v>
+      </c>
+      <c r="I30" s="49" t="s">
         <v>175</v>
       </c>
       <c r="J30" s="2" t="s">
@@ -3791,172 +3865,174 @@
       <c r="K30" s="1">
         <v>6</v>
       </c>
-      <c r="L30" s="67">
+      <c r="L30" s="66">
         <v>1</v>
       </c>
-      <c r="M30" s="52">
+      <c r="M30" s="51">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N30" s="71" t="s">
+      <c r="N30" s="70" t="s">
         <v>189</v>
       </c>
-      <c r="O30" s="54">
+      <c r="O30" s="53">
         <v>3.8355999999999999</v>
       </c>
-      <c r="P30" s="55">
+      <c r="P30" s="54">
         <f t="shared" si="1"/>
         <v>3.8355999999999999</v>
       </c>
-      <c r="Q30" s="55">
+      <c r="Q30" s="54">
         <f t="shared" si="2"/>
         <v>23.0136</v>
       </c>
-      <c r="R30" s="54">
+      <c r="R30" s="53">
         <v>3.8355999999999999</v>
       </c>
-      <c r="S30" s="55">
+      <c r="S30" s="54">
         <f t="shared" si="3"/>
         <v>19.178000000000001</v>
       </c>
-      <c r="T30" s="56"/>
+      <c r="T30" s="55"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
     </row>
     <row r="31" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="33">
+      <c r="A31" s="32">
         <v>29</v>
       </c>
-      <c r="B31" s="113"/>
-      <c r="C31" s="18" t="s">
+      <c r="B31" s="110"/>
+      <c r="C31" s="128" t="s">
         <v>133</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="129" t="s">
         <v>134</v>
       </c>
-      <c r="E31" s="17" t="s">
+      <c r="E31" s="129" t="s">
         <v>135</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F31" s="129" t="s">
         <v>133</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="130" t="s">
         <v>136</v>
       </c>
-      <c r="H31" s="37" t="s">
-        <v>216</v>
-      </c>
-      <c r="I31" s="37" t="s">
+      <c r="H31" s="131" t="s">
+        <v>215</v>
+      </c>
+      <c r="I31" s="131" t="s">
         <v>175</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="J31" s="130" t="s">
         <v>175</v>
       </c>
-      <c r="K31" s="39">
+      <c r="K31" s="132">
         <v>6</v>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="133">
         <v>1</v>
       </c>
-      <c r="M31" s="39">
+      <c r="M31" s="132">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N31" s="57" t="s">
+      <c r="N31" s="134" t="s">
         <v>189</v>
       </c>
-      <c r="O31" s="40">
+      <c r="O31" s="135">
         <v>15.131399999999999</v>
       </c>
-      <c r="P31" s="41">
+      <c r="P31" s="136">
         <f t="shared" si="1"/>
         <v>15.131399999999999</v>
       </c>
-      <c r="Q31" s="41">
+      <c r="Q31" s="136">
         <f t="shared" si="2"/>
         <v>90.788399999999996</v>
       </c>
-      <c r="R31" s="40">
+      <c r="R31" s="135">
         <v>15.131399999999999</v>
       </c>
-      <c r="S31" s="41">
+      <c r="S31" s="136">
         <f t="shared" si="3"/>
         <v>75.656999999999996</v>
       </c>
-      <c r="T31" s="49"/>
+      <c r="T31" s="48" t="s">
+        <v>245</v>
+      </c>
       <c r="U31" s="3"/>
       <c r="V31" s="3"/>
     </row>
     <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="33">
+      <c r="A32" s="32">
         <v>30</v>
       </c>
-      <c r="B32" s="113"/>
-      <c r="C32" s="18" t="s">
+      <c r="B32" s="110"/>
+      <c r="C32" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="D32" s="17" t="s">
+      <c r="D32" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="E32" s="17" t="s">
+      <c r="E32" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F32" s="16" t="s">
         <v>140</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H32" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="I32" s="38" t="s">
+      <c r="H32" s="36" t="s">
+        <v>216</v>
+      </c>
+      <c r="I32" s="37" t="s">
         <v>175</v>
       </c>
       <c r="J32" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="K32" s="39">
+      <c r="K32" s="38">
         <v>6</v>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="14">
         <v>1</v>
       </c>
-      <c r="M32" s="39">
+      <c r="M32" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N32" s="57" t="s">
+      <c r="N32" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O32" s="40">
+      <c r="O32" s="39">
         <v>0.30049999999999999</v>
       </c>
-      <c r="P32" s="41">
+      <c r="P32" s="40">
         <f t="shared" si="1"/>
         <v>0.30049999999999999</v>
       </c>
-      <c r="Q32" s="41">
+      <c r="Q32" s="40">
         <f t="shared" si="2"/>
         <v>1.8029999999999999</v>
       </c>
-      <c r="R32" s="40">
+      <c r="R32" s="39">
         <v>0.30049999999999999</v>
       </c>
-      <c r="S32" s="41">
+      <c r="S32" s="40">
         <f t="shared" si="3"/>
         <v>1.5024999999999999</v>
       </c>
-      <c r="T32" s="49"/>
+      <c r="T32" s="48"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
     </row>
     <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="33">
+      <c r="A33" s="32">
         <v>31</v>
       </c>
-      <c r="B33" s="113"/>
-      <c r="C33" s="16" t="s">
+      <c r="B33" s="110"/>
+      <c r="C33" s="15" t="s">
         <v>141</v>
       </c>
       <c r="D33" s="6" t="s">
@@ -3971,72 +4047,72 @@
       <c r="G33" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="H33" s="37" t="s">
-        <v>218</v>
-      </c>
-      <c r="I33" s="51" t="s">
+      <c r="H33" s="36" t="s">
+        <v>217</v>
+      </c>
+      <c r="I33" s="50" t="s">
         <v>175</v>
       </c>
       <c r="J33" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="K33" s="39">
+      <c r="K33" s="38">
         <v>25</v>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="14">
         <v>4</v>
       </c>
-      <c r="M33" s="39">
+      <c r="M33" s="38">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N33" s="57" t="s">
+      <c r="N33" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O33" s="40">
+      <c r="O33" s="39">
         <v>0.26579999999999998</v>
       </c>
-      <c r="P33" s="41">
+      <c r="P33" s="40">
         <f t="shared" si="1"/>
         <v>1.0631999999999999</v>
       </c>
-      <c r="Q33" s="41">
+      <c r="Q33" s="40">
         <f t="shared" si="2"/>
         <v>6.6449999999999996</v>
       </c>
-      <c r="R33" s="40">
+      <c r="R33" s="39">
         <v>0.26579999999999998</v>
       </c>
-      <c r="S33" s="41">
+      <c r="S33" s="40">
         <f t="shared" si="3"/>
         <v>5.3159999999999998</v>
       </c>
-      <c r="T33" s="49"/>
+      <c r="T33" s="48"/>
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
     </row>
     <row r="34" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="33">
+      <c r="A34" s="32">
         <v>32</v>
       </c>
-      <c r="B34" s="113"/>
-      <c r="C34" s="18" t="s">
+      <c r="B34" s="110"/>
+      <c r="C34" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="D34" s="17" t="s">
+      <c r="D34" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E34" s="17" t="s">
+      <c r="E34" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" s="16" t="s">
         <v>148</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="H34" s="37" t="s">
-        <v>219</v>
+      <c r="H34" s="36" t="s">
+        <v>218</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>175</v>
@@ -4044,62 +4120,62 @@
       <c r="J34" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="K34" s="39">
+      <c r="K34" s="38">
         <v>6</v>
       </c>
-      <c r="L34" s="15">
+      <c r="L34" s="14">
         <v>1</v>
       </c>
-      <c r="M34" s="39">
+      <c r="M34" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N34" s="57" t="s">
+      <c r="N34" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="O34" s="40">
+      <c r="O34" s="39">
         <v>1.0964</v>
       </c>
-      <c r="P34" s="41">
+      <c r="P34" s="40">
         <f t="shared" si="1"/>
         <v>1.0964</v>
       </c>
-      <c r="Q34" s="41">
+      <c r="Q34" s="40">
         <f t="shared" si="2"/>
         <v>6.5784000000000002</v>
       </c>
-      <c r="R34" s="40">
+      <c r="R34" s="39">
         <v>1.0964</v>
       </c>
-      <c r="S34" s="41">
+      <c r="S34" s="40">
         <f t="shared" si="3"/>
         <v>5.4820000000000002</v>
       </c>
-      <c r="T34" s="49"/>
+      <c r="T34" s="48"/>
       <c r="U34" s="3"/>
       <c r="V34" s="3"/>
     </row>
     <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="33">
+      <c r="A35" s="32">
         <v>33</v>
       </c>
-      <c r="B35" s="114"/>
-      <c r="C35" s="107" t="s">
+      <c r="B35" s="111"/>
+      <c r="C35" s="104" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="104" t="s">
+      <c r="D35" s="101" t="s">
         <v>150</v>
       </c>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="45" t="s">
         <v>151</v>
       </c>
-      <c r="F35" s="104" t="s">
+      <c r="F35" s="101" t="s">
         <v>152</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="H35" s="60" t="s">
+      <c r="H35" s="59" t="s">
         <v>175</v>
       </c>
       <c r="I35" s="8" t="s">
@@ -4108,65 +4184,65 @@
       <c r="J35" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="K35" s="45">
+      <c r="K35" s="44">
         <v>30</v>
       </c>
-      <c r="L35" s="108">
+      <c r="L35" s="105">
         <v>5</v>
       </c>
-      <c r="M35" s="45">
+      <c r="M35" s="44">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N35" s="109" t="s">
-        <v>241</v>
-      </c>
-      <c r="O35" s="42">
+      <c r="N35" s="106" t="s">
+        <v>240</v>
+      </c>
+      <c r="O35" s="41">
         <v>0.46200000000000002</v>
       </c>
-      <c r="P35" s="43">
+      <c r="P35" s="42">
         <f t="shared" si="1"/>
         <v>2.31</v>
       </c>
-      <c r="Q35" s="43">
+      <c r="Q35" s="42">
         <f t="shared" si="2"/>
         <v>13.860000000000001</v>
       </c>
-      <c r="R35" s="42">
+      <c r="R35" s="41">
         <v>0.46200000000000002</v>
       </c>
-      <c r="S35" s="43">
+      <c r="S35" s="42">
         <f t="shared" si="3"/>
         <v>11.55</v>
       </c>
-      <c r="T35" s="62"/>
+      <c r="T35" s="61"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
     </row>
     <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="33">
+      <c r="A36" s="32">
         <v>34</v>
       </c>
-      <c r="B36" s="112" t="s">
+      <c r="B36" s="109" t="s">
         <v>24</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="D36" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="E36" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F36" s="14" t="s">
+      <c r="F36" s="13" t="s">
         <v>156</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="H36" s="50" t="s">
-        <v>220</v>
+      <c r="H36" s="49" t="s">
+        <v>219</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>175</v>
@@ -4174,63 +4250,63 @@
       <c r="J36" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="K36" s="52">
+      <c r="K36" s="51">
         <v>30</v>
       </c>
-      <c r="L36" s="67">
+      <c r="L36" s="66">
         <v>5</v>
       </c>
-      <c r="M36" s="52">
+      <c r="M36" s="51">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="N36" s="71" t="s">
+      <c r="N36" s="70" t="s">
         <v>189</v>
       </c>
-      <c r="O36" s="75">
+      <c r="O36" s="73">
         <v>9.2399999999999996E-2</v>
       </c>
-      <c r="P36" s="55">
+      <c r="P36" s="54">
         <f t="shared" si="1"/>
         <v>0.46199999999999997</v>
       </c>
-      <c r="Q36" s="55">
+      <c r="Q36" s="54">
         <f t="shared" si="2"/>
         <v>2.7719999999999998</v>
       </c>
-      <c r="R36" s="75">
+      <c r="R36" s="73">
         <v>9.2399999999999996E-2</v>
       </c>
-      <c r="S36" s="55">
+      <c r="S36" s="54">
         <f t="shared" si="3"/>
         <v>2.31</v>
       </c>
-      <c r="T36" s="72"/>
+      <c r="T36" s="71"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
     </row>
     <row r="37" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="33">
+      <c r="A37" s="32">
         <v>35</v>
       </c>
-      <c r="B37" s="113"/>
-      <c r="C37" s="18" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E37" s="17" t="s">
+      <c r="E37" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" s="16" t="s">
         <v>159</v>
       </c>
       <c r="G37" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="H37" s="36" t="s">
         <v>221</v>
-      </c>
-      <c r="H37" s="37" t="s">
-        <v>222</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>175</v>
@@ -4238,125 +4314,125 @@
       <c r="J37" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="K37" s="39">
+      <c r="K37" s="38">
         <v>7</v>
       </c>
-      <c r="L37" s="15">
+      <c r="L37" s="14">
         <v>1</v>
       </c>
-      <c r="M37" s="39">
+      <c r="M37" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N37" s="59" t="s">
+      <c r="N37" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="O37" s="40">
+      <c r="O37" s="39">
         <v>0.25</v>
       </c>
-      <c r="P37" s="41">
+      <c r="P37" s="40">
         <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
-      <c r="Q37" s="41">
+      <c r="Q37" s="40">
         <f t="shared" si="2"/>
         <v>1.75</v>
       </c>
-      <c r="R37" s="40">
+      <c r="R37" s="39">
         <v>0.25</v>
       </c>
-      <c r="S37" s="41">
+      <c r="S37" s="40">
         <f t="shared" si="3"/>
         <v>1.25</v>
       </c>
-      <c r="T37" s="49"/>
+      <c r="T37" s="48"/>
       <c r="U37" s="3"/>
       <c r="V37" s="3"/>
     </row>
     <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="33">
+      <c r="A38" s="32">
         <v>36</v>
       </c>
-      <c r="B38" s="113"/>
-      <c r="C38" s="18" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F38" s="17" t="s">
-        <v>234</v>
+      <c r="F38" s="16" t="s">
+        <v>233</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="H38" s="37" t="s">
-        <v>233</v>
+        <v>241</v>
+      </c>
+      <c r="H38" s="36" t="s">
+        <v>232</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K38" s="39">
+      <c r="K38" s="38">
         <v>7</v>
       </c>
-      <c r="L38" s="15">
+      <c r="L38" s="14">
         <v>1</v>
       </c>
-      <c r="M38" s="39">
+      <c r="M38" s="38">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N38" s="59" t="s">
+      <c r="N38" s="94" t="s">
         <v>189</v>
       </c>
-      <c r="O38" s="40">
+      <c r="O38" s="39">
         <v>0.1804</v>
       </c>
-      <c r="P38" s="41">
+      <c r="P38" s="40">
         <f t="shared" si="1"/>
         <v>0.1804</v>
       </c>
-      <c r="Q38" s="41">
+      <c r="Q38" s="40">
         <f t="shared" si="2"/>
         <v>1.2627999999999999</v>
       </c>
-      <c r="R38" s="40">
+      <c r="R38" s="39">
         <v>0.14430000000000001</v>
       </c>
-      <c r="S38" s="41">
+      <c r="S38" s="40">
         <f t="shared" si="3"/>
         <v>0.72150000000000003</v>
       </c>
-      <c r="T38" s="49"/>
+      <c r="T38" s="48"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
     </row>
     <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="111">
+      <c r="A39" s="108">
         <v>37</v>
       </c>
-      <c r="B39" s="114"/>
-      <c r="C39" s="70" t="s">
+      <c r="B39" s="111"/>
+      <c r="C39" s="69" t="s">
         <v>163</v>
       </c>
-      <c r="D39" s="68" t="s">
+      <c r="D39" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="E39" s="68" t="s">
+      <c r="E39" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="F39" s="68" t="s">
+      <c r="F39" s="67" t="s">
         <v>165</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="H39" s="60" t="s">
-        <v>226</v>
+      <c r="H39" s="59" t="s">
+        <v>225</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>175</v>
@@ -4364,108 +4440,108 @@
       <c r="J39" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="K39" s="45">
+      <c r="K39" s="44">
         <v>7</v>
       </c>
-      <c r="L39" s="69">
+      <c r="L39" s="68">
         <v>1</v>
       </c>
-      <c r="M39" s="45">
+      <c r="M39" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N39" s="65" t="s">
+      <c r="N39" s="64" t="s">
         <v>189</v>
       </c>
-      <c r="O39" s="42">
+      <c r="O39" s="41">
         <v>0.22420000000000001</v>
       </c>
-      <c r="P39" s="43">
+      <c r="P39" s="42">
         <f t="shared" si="1"/>
         <v>0.22420000000000001</v>
       </c>
-      <c r="Q39" s="43">
+      <c r="Q39" s="42">
         <f t="shared" si="2"/>
         <v>1.5694000000000001</v>
       </c>
-      <c r="R39" s="42">
+      <c r="R39" s="41">
         <v>0.22420000000000001</v>
       </c>
-      <c r="S39" s="43">
+      <c r="S39" s="42">
         <f t="shared" si="3"/>
         <v>1.121</v>
       </c>
-      <c r="T39" s="44"/>
+      <c r="T39" s="43"/>
       <c r="U39" s="3"/>
       <c r="V39" s="3"/>
     </row>
     <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="26"/>
-      <c r="K40" s="26"/>
-      <c r="L40" s="119" t="s">
+      <c r="H40" s="25"/>
+      <c r="I40" s="25"/>
+      <c r="J40" s="25"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="116" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="119"/>
-      <c r="N40" s="119"/>
-      <c r="O40" s="119"/>
-      <c r="P40" s="30"/>
-      <c r="Q40" s="30">
+      <c r="M40" s="116"/>
+      <c r="N40" s="116"/>
+      <c r="O40" s="116"/>
+      <c r="P40" s="29"/>
+      <c r="Q40" s="29">
         <f>SUM(Q3:Q39)</f>
-        <v>199.66589999999999</v>
-      </c>
-      <c r="R40" s="30"/>
-      <c r="S40" s="22">
+        <v>200.0187</v>
+      </c>
+      <c r="R40" s="29"/>
+      <c r="S40" s="21">
         <f>SUM(S3:S39)</f>
-        <v>154.76600000000002</v>
-      </c>
-      <c r="T40" s="26"/>
+        <v>155.01500000000001</v>
+      </c>
+      <c r="T40" s="25"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="28"/>
-      <c r="K41" s="26"/>
-      <c r="L41" s="115" t="s">
+      <c r="H41" s="25"/>
+      <c r="I41" s="25"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="112" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="115"/>
-      <c r="N41" s="115"/>
-      <c r="O41" s="115"/>
-      <c r="P41" s="22">
+      <c r="M41" s="112"/>
+      <c r="N41" s="112"/>
+      <c r="O41" s="112"/>
+      <c r="P41" s="21">
         <f>SUM(P3:P39)</f>
-        <v>31.930699999999991</v>
-      </c>
-      <c r="Q41" s="22">
+        <v>31.980499999999996</v>
+      </c>
+      <c r="Q41" s="21">
         <f>Q40/5</f>
-        <v>39.93318</v>
-      </c>
-      <c r="R41" s="27"/>
-      <c r="S41" s="29">
+        <v>40.003740000000001</v>
+      </c>
+      <c r="R41" s="26"/>
+      <c r="S41" s="28">
         <f>S40/5</f>
-        <v>30.953200000000002</v>
-      </c>
-      <c r="T41" s="26"/>
+        <v>31.003000000000004</v>
+      </c>
+      <c r="T41" s="25"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I42" s="24"/>
-      <c r="J42" s="24"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="J43" s="23"/>
+      <c r="J43" s="22"/>
       <c r="U43" s="3"/>
       <c r="V43" s="3"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I44" s="24"/>
-      <c r="J44" s="24"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23"/>
       <c r="U44" s="3"/>
       <c r="V44" s="3"/>
     </row>
@@ -4699,45 +4775,46 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N8" r:id="rId1"/>
-    <hyperlink ref="N3" r:id="rId2"/>
-    <hyperlink ref="N4" r:id="rId3"/>
-    <hyperlink ref="N5" r:id="rId4"/>
-    <hyperlink ref="N6" r:id="rId5"/>
-    <hyperlink ref="N7" r:id="rId6"/>
-    <hyperlink ref="N9" r:id="rId7"/>
-    <hyperlink ref="N10" r:id="rId8"/>
-    <hyperlink ref="N12" r:id="rId9"/>
-    <hyperlink ref="N14" r:id="rId10"/>
-    <hyperlink ref="N16" r:id="rId11"/>
-    <hyperlink ref="N17" r:id="rId12"/>
-    <hyperlink ref="N18" r:id="rId13"/>
-    <hyperlink ref="N19" r:id="rId14"/>
-    <hyperlink ref="N20" r:id="rId15"/>
-    <hyperlink ref="N22" r:id="rId16"/>
-    <hyperlink ref="N23" r:id="rId17"/>
-    <hyperlink ref="N24" r:id="rId18"/>
-    <hyperlink ref="N25" r:id="rId19"/>
-    <hyperlink ref="N26" r:id="rId20"/>
-    <hyperlink ref="N27" r:id="rId21"/>
-    <hyperlink ref="N28" r:id="rId22"/>
-    <hyperlink ref="N29" r:id="rId23"/>
-    <hyperlink ref="N30" r:id="rId24"/>
-    <hyperlink ref="N31" r:id="rId25"/>
-    <hyperlink ref="N32" r:id="rId26"/>
-    <hyperlink ref="N33" r:id="rId27"/>
-    <hyperlink ref="N34" r:id="rId28"/>
-    <hyperlink ref="N36" r:id="rId29"/>
-    <hyperlink ref="N37" r:id="rId30"/>
-    <hyperlink ref="N21" r:id="rId31"/>
-    <hyperlink ref="N39" r:id="rId32"/>
-    <hyperlink ref="N11" r:id="rId33"/>
-    <hyperlink ref="N13" r:id="rId34"/>
-    <hyperlink ref="N15" r:id="rId35"/>
-    <hyperlink ref="N35" r:id="rId36"/>
+    <hyperlink ref="N8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N17" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N22" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N32" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N33" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="N34" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="N36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="N37" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="N21" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="N39" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="N11" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="N13" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="N15" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="N35" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="N38" r:id="rId37" xr:uid="{08CAC2E9-2AE0-4129-B0E5-392E22FB012A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId38"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
quote from Karen has been added to LCSC BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOM_LCSC.xlsx
+++ b/Deliverables/BOM/BOM_LCSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDA3C3B-D461-4ED2-B074-3AE9D842EB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F840EA54-61D1-41F3-95EC-227217F41A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="247">
   <si>
     <t>S. No.</t>
   </si>
@@ -780,6 +780,9 @@
   </si>
   <si>
     <t>Out of stock on LCSC</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
   </si>
 </sst>
 </file>
@@ -1613,6 +1616,66 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1636,66 +1699,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1994,7 +1997,7 @@
     <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.5703125" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="21" bestFit="1" customWidth="1"/>
@@ -2003,28 +2006,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="133" t="s">
         <v>239</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114"/>
-      <c r="I1" s="114"/>
-      <c r="J1" s="114"/>
-      <c r="K1" s="114"/>
-      <c r="L1" s="114"/>
-      <c r="M1" s="114"/>
-      <c r="N1" s="114"/>
-      <c r="O1" s="114"/>
-      <c r="P1" s="114"/>
-      <c r="Q1" s="114"/>
-      <c r="R1" s="114"/>
-      <c r="S1" s="114"/>
-      <c r="T1" s="115"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
+      <c r="J1" s="134"/>
+      <c r="K1" s="134"/>
+      <c r="L1" s="134"/>
+      <c r="M1" s="134"/>
+      <c r="N1" s="134"/>
+      <c r="O1" s="134"/>
+      <c r="P1" s="134"/>
+      <c r="Q1" s="134"/>
+      <c r="R1" s="134"/>
+      <c r="S1" s="134"/>
+      <c r="T1" s="135"/>
     </row>
     <row r="2" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
@@ -2092,7 +2095,7 @@
       <c r="A3" s="32">
         <v>1</v>
       </c>
-      <c r="B3" s="109" t="s">
+      <c r="B3" s="129" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="12" t="s">
@@ -2158,7 +2161,7 @@
       <c r="A4" s="32">
         <v>2</v>
       </c>
-      <c r="B4" s="110"/>
+      <c r="B4" s="130"/>
       <c r="C4" s="17" t="s">
         <v>34</v>
       </c>
@@ -2222,7 +2225,7 @@
       <c r="A5" s="32">
         <v>3</v>
       </c>
-      <c r="B5" s="110"/>
+      <c r="B5" s="130"/>
       <c r="C5" s="17" t="s">
         <v>39</v>
       </c>
@@ -2286,7 +2289,7 @@
       <c r="A6" s="32">
         <v>4</v>
       </c>
-      <c r="B6" s="110"/>
+      <c r="B6" s="130"/>
       <c r="C6" s="17" t="s">
         <v>43</v>
       </c>
@@ -2350,7 +2353,7 @@
       <c r="A7" s="32">
         <v>5</v>
       </c>
-      <c r="B7" s="110"/>
+      <c r="B7" s="130"/>
       <c r="C7" s="17" t="s">
         <v>46</v>
       </c>
@@ -2414,7 +2417,7 @@
       <c r="A8" s="32">
         <v>6</v>
       </c>
-      <c r="B8" s="110"/>
+      <c r="B8" s="130"/>
       <c r="C8" s="17" t="s">
         <v>49</v>
       </c>
@@ -2478,7 +2481,7 @@
       <c r="A9" s="32">
         <v>7</v>
       </c>
-      <c r="B9" s="110"/>
+      <c r="B9" s="130"/>
       <c r="C9" s="15" t="s">
         <v>54</v>
       </c>
@@ -2542,7 +2545,7 @@
       <c r="A10" s="32">
         <v>8</v>
       </c>
-      <c r="B10" s="110"/>
+      <c r="B10" s="130"/>
       <c r="C10" s="17" t="s">
         <v>57</v>
       </c>
@@ -2606,7 +2609,7 @@
       <c r="A11" s="32">
         <v>9</v>
       </c>
-      <c r="B11" s="110"/>
+      <c r="B11" s="130"/>
       <c r="C11" s="17" t="s">
         <v>61</v>
       </c>
@@ -2669,7 +2672,7 @@
       <c r="A12" s="32">
         <v>10</v>
       </c>
-      <c r="B12" s="111"/>
+      <c r="B12" s="131"/>
       <c r="C12" s="69" t="s">
         <v>64</v>
       </c>
@@ -2733,7 +2736,7 @@
       <c r="A13" s="32">
         <v>11</v>
       </c>
-      <c r="B13" s="109" t="s">
+      <c r="B13" s="129" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -2799,7 +2802,7 @@
       <c r="A14" s="32">
         <v>12</v>
       </c>
-      <c r="B14" s="111"/>
+      <c r="B14" s="131"/>
       <c r="C14" s="72" t="s">
         <v>73</v>
       </c>
@@ -2993,7 +2996,7 @@
       <c r="A17" s="32">
         <v>15</v>
       </c>
-      <c r="B17" s="109" t="s">
+      <c r="B17" s="129" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="12" t="s">
@@ -3059,7 +3062,7 @@
       <c r="A18" s="32">
         <v>16</v>
       </c>
-      <c r="B18" s="110"/>
+      <c r="B18" s="130"/>
       <c r="C18" s="17" t="s">
         <v>90</v>
       </c>
@@ -3123,7 +3126,7 @@
       <c r="A19" s="32">
         <v>17</v>
       </c>
-      <c r="B19" s="110"/>
+      <c r="B19" s="130"/>
       <c r="C19" s="17" t="s">
         <v>94</v>
       </c>
@@ -3187,7 +3190,7 @@
       <c r="A20" s="32">
         <v>18</v>
       </c>
-      <c r="B20" s="110"/>
+      <c r="B20" s="130"/>
       <c r="C20" s="17" t="s">
         <v>97</v>
       </c>
@@ -3251,7 +3254,7 @@
       <c r="A21" s="32">
         <v>19</v>
       </c>
-      <c r="B21" s="110"/>
+      <c r="B21" s="130"/>
       <c r="C21" s="15" t="s">
         <v>237</v>
       </c>
@@ -3315,7 +3318,7 @@
       <c r="A22" s="32">
         <v>20</v>
       </c>
-      <c r="B22" s="110"/>
+      <c r="B22" s="130"/>
       <c r="C22" s="17" t="s">
         <v>101</v>
       </c>
@@ -3379,7 +3382,7 @@
       <c r="A23" s="32">
         <v>21</v>
       </c>
-      <c r="B23" s="110"/>
+      <c r="B23" s="130"/>
       <c r="C23" s="17" t="s">
         <v>104</v>
       </c>
@@ -3443,7 +3446,7 @@
       <c r="A24" s="32">
         <v>22</v>
       </c>
-      <c r="B24" s="110"/>
+      <c r="B24" s="130"/>
       <c r="C24" s="17" t="s">
         <v>107</v>
       </c>
@@ -3507,7 +3510,7 @@
       <c r="A25" s="32">
         <v>23</v>
       </c>
-      <c r="B25" s="111"/>
+      <c r="B25" s="131"/>
       <c r="C25" s="69" t="s">
         <v>110</v>
       </c>
@@ -3571,63 +3574,63 @@
       <c r="A26" s="32">
         <v>24</v>
       </c>
-      <c r="B26" s="109" t="s">
+      <c r="B26" s="129" t="s">
         <v>190</v>
       </c>
-      <c r="C26" s="126" t="s">
+      <c r="C26" s="118" t="s">
         <v>113</v>
       </c>
-      <c r="D26" s="118" t="s">
+      <c r="D26" s="110" t="s">
         <v>114</v>
       </c>
-      <c r="E26" s="118" t="s">
+      <c r="E26" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="118" t="s">
+      <c r="F26" s="110" t="s">
         <v>115</v>
       </c>
-      <c r="G26" s="119" t="s">
+      <c r="G26" s="111" t="s">
         <v>116</v>
       </c>
-      <c r="H26" s="120" t="s">
+      <c r="H26" s="112" t="s">
         <v>229</v>
       </c>
-      <c r="I26" s="119" t="s">
+      <c r="I26" s="111" t="s">
         <v>175</v>
       </c>
-      <c r="J26" s="119" t="s">
+      <c r="J26" s="111" t="s">
         <v>175</v>
       </c>
-      <c r="K26" s="119">
+      <c r="K26" s="111">
         <v>12</v>
       </c>
-      <c r="L26" s="122">
+      <c r="L26" s="114">
         <v>2</v>
       </c>
-      <c r="M26" s="123">
+      <c r="M26" s="115">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N26" s="127" t="s">
-        <v>189</v>
-      </c>
-      <c r="O26" s="124">
-        <v>0.88370000000000004</v>
-      </c>
-      <c r="P26" s="125">
+      <c r="N26" s="119" t="s">
+        <v>246</v>
+      </c>
+      <c r="O26" s="116">
+        <v>1.5</v>
+      </c>
+      <c r="P26" s="117">
         <f t="shared" si="1"/>
-        <v>1.7674000000000001</v>
-      </c>
-      <c r="Q26" s="125">
+        <v>3</v>
+      </c>
+      <c r="Q26" s="117">
         <f t="shared" si="2"/>
-        <v>10.6044</v>
-      </c>
-      <c r="R26" s="124">
-        <v>0.65820000000000001</v>
-      </c>
-      <c r="S26" s="125">
+        <v>18</v>
+      </c>
+      <c r="R26" s="116">
+        <v>1.5</v>
+      </c>
+      <c r="S26" s="117">
         <f t="shared" si="3"/>
-        <v>6.5819999999999999</v>
+        <v>15</v>
       </c>
       <c r="T26" s="55" t="s">
         <v>245</v>
@@ -3639,7 +3642,7 @@
       <c r="A27" s="32">
         <v>25</v>
       </c>
-      <c r="B27" s="111"/>
+      <c r="B27" s="131"/>
       <c r="C27" s="72" t="s">
         <v>117</v>
       </c>
@@ -3703,61 +3706,61 @@
       <c r="A28" s="32">
         <v>26</v>
       </c>
-      <c r="B28" s="109" t="s">
+      <c r="B28" s="129" t="s">
         <v>191</v>
       </c>
-      <c r="C28" s="117" t="s">
+      <c r="C28" s="109" t="s">
         <v>121</v>
       </c>
-      <c r="D28" s="118" t="s">
+      <c r="D28" s="110" t="s">
         <v>122</v>
       </c>
-      <c r="E28" s="118" t="s">
+      <c r="E28" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="F28" s="118" t="s">
+      <c r="F28" s="110" t="s">
         <v>123</v>
       </c>
-      <c r="G28" s="119" t="s">
+      <c r="G28" s="111" t="s">
         <v>120</v>
       </c>
-      <c r="H28" s="120" t="s">
+      <c r="H28" s="112" t="s">
         <v>242</v>
       </c>
-      <c r="I28" s="119" t="s">
+      <c r="I28" s="111" t="s">
         <v>243</v>
       </c>
-      <c r="J28" s="121" t="s">
+      <c r="J28" s="113" t="s">
         <v>186</v>
       </c>
-      <c r="K28" s="119">
+      <c r="K28" s="111">
         <v>7</v>
       </c>
-      <c r="L28" s="122">
+      <c r="L28" s="114">
         <v>1</v>
       </c>
-      <c r="M28" s="123">
+      <c r="M28" s="115">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N28" s="127" t="s">
+      <c r="N28" s="119" t="s">
         <v>189</v>
       </c>
-      <c r="O28" s="124">
+      <c r="O28" s="116">
         <v>0.56630000000000003</v>
       </c>
-      <c r="P28" s="125">
+      <c r="P28" s="117">
         <f t="shared" si="1"/>
         <v>0.56630000000000003</v>
       </c>
-      <c r="Q28" s="125">
+      <c r="Q28" s="117">
         <f t="shared" si="2"/>
         <v>3.9641000000000002</v>
       </c>
-      <c r="R28" s="124">
+      <c r="R28" s="116">
         <v>0.56630000000000003</v>
       </c>
-      <c r="S28" s="125">
+      <c r="S28" s="117">
         <f t="shared" si="3"/>
         <v>2.8315000000000001</v>
       </c>
@@ -3771,7 +3774,7 @@
       <c r="A29" s="32">
         <v>27</v>
       </c>
-      <c r="B29" s="111"/>
+      <c r="B29" s="131"/>
       <c r="C29" s="72" t="s">
         <v>124</v>
       </c>
@@ -3835,7 +3838,7 @@
       <c r="A30" s="32">
         <v>28</v>
       </c>
-      <c r="B30" s="109" t="s">
+      <c r="B30" s="129" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="12" t="s">
@@ -3901,61 +3904,61 @@
       <c r="A31" s="32">
         <v>29</v>
       </c>
-      <c r="B31" s="110"/>
-      <c r="C31" s="128" t="s">
+      <c r="B31" s="130"/>
+      <c r="C31" s="120" t="s">
         <v>133</v>
       </c>
-      <c r="D31" s="129" t="s">
+      <c r="D31" s="121" t="s">
         <v>134</v>
       </c>
-      <c r="E31" s="129" t="s">
+      <c r="E31" s="121" t="s">
         <v>135</v>
       </c>
-      <c r="F31" s="129" t="s">
+      <c r="F31" s="121" t="s">
         <v>133</v>
       </c>
-      <c r="G31" s="130" t="s">
+      <c r="G31" s="122" t="s">
         <v>136</v>
       </c>
-      <c r="H31" s="131" t="s">
+      <c r="H31" s="123" t="s">
         <v>215</v>
       </c>
-      <c r="I31" s="131" t="s">
+      <c r="I31" s="123" t="s">
         <v>175</v>
       </c>
-      <c r="J31" s="130" t="s">
+      <c r="J31" s="122" t="s">
         <v>175</v>
       </c>
-      <c r="K31" s="132">
+      <c r="K31" s="124">
         <v>6</v>
       </c>
-      <c r="L31" s="133">
+      <c r="L31" s="125">
         <v>1</v>
       </c>
-      <c r="M31" s="132">
+      <c r="M31" s="124">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N31" s="134" t="s">
-        <v>189</v>
-      </c>
-      <c r="O31" s="135">
-        <v>15.131399999999999</v>
-      </c>
-      <c r="P31" s="136">
+      <c r="N31" s="126" t="s">
+        <v>246</v>
+      </c>
+      <c r="O31" s="127">
+        <v>8.57</v>
+      </c>
+      <c r="P31" s="128">
         <f t="shared" si="1"/>
-        <v>15.131399999999999</v>
-      </c>
-      <c r="Q31" s="136">
+        <v>8.57</v>
+      </c>
+      <c r="Q31" s="128">
         <f t="shared" si="2"/>
-        <v>90.788399999999996</v>
-      </c>
-      <c r="R31" s="135">
-        <v>15.131399999999999</v>
-      </c>
-      <c r="S31" s="136">
+        <v>51.42</v>
+      </c>
+      <c r="R31" s="127">
+        <v>8.57</v>
+      </c>
+      <c r="S31" s="128">
         <f t="shared" si="3"/>
-        <v>75.656999999999996</v>
+        <v>42.85</v>
       </c>
       <c r="T31" s="48" t="s">
         <v>245</v>
@@ -3967,7 +3970,7 @@
       <c r="A32" s="32">
         <v>30</v>
       </c>
-      <c r="B32" s="110"/>
+      <c r="B32" s="130"/>
       <c r="C32" s="17" t="s">
         <v>137</v>
       </c>
@@ -4031,7 +4034,7 @@
       <c r="A33" s="32">
         <v>31</v>
       </c>
-      <c r="B33" s="110"/>
+      <c r="B33" s="130"/>
       <c r="C33" s="15" t="s">
         <v>141</v>
       </c>
@@ -4095,7 +4098,7 @@
       <c r="A34" s="32">
         <v>32</v>
       </c>
-      <c r="B34" s="110"/>
+      <c r="B34" s="130"/>
       <c r="C34" s="17" t="s">
         <v>145</v>
       </c>
@@ -4159,7 +4162,7 @@
       <c r="A35" s="32">
         <v>33</v>
       </c>
-      <c r="B35" s="111"/>
+      <c r="B35" s="131"/>
       <c r="C35" s="104" t="s">
         <v>149</v>
       </c>
@@ -4223,7 +4226,7 @@
       <c r="A36" s="32">
         <v>34</v>
       </c>
-      <c r="B36" s="109" t="s">
+      <c r="B36" s="129" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="12" t="s">
@@ -4289,7 +4292,7 @@
       <c r="A37" s="32">
         <v>35</v>
       </c>
-      <c r="B37" s="110"/>
+      <c r="B37" s="130"/>
       <c r="C37" s="17" t="s">
         <v>157</v>
       </c>
@@ -4353,7 +4356,7 @@
       <c r="A38" s="32">
         <v>36</v>
       </c>
-      <c r="B38" s="110"/>
+      <c r="B38" s="130"/>
       <c r="C38" s="17" t="s">
         <v>160</v>
       </c>
@@ -4415,7 +4418,7 @@
       <c r="A39" s="108">
         <v>37</v>
       </c>
-      <c r="B39" s="111"/>
+      <c r="B39" s="131"/>
       <c r="C39" s="69" t="s">
         <v>163</v>
       </c>
@@ -4480,21 +4483,21 @@
       <c r="I40" s="25"/>
       <c r="J40" s="25"/>
       <c r="K40" s="25"/>
-      <c r="L40" s="116" t="s">
+      <c r="L40" s="136" t="s">
         <v>25</v>
       </c>
-      <c r="M40" s="116"/>
-      <c r="N40" s="116"/>
-      <c r="O40" s="116"/>
+      <c r="M40" s="136"/>
+      <c r="N40" s="136"/>
+      <c r="O40" s="136"/>
       <c r="P40" s="29"/>
       <c r="Q40" s="29">
         <f>SUM(Q3:Q39)</f>
-        <v>200.0187</v>
+        <v>168.04589999999999</v>
       </c>
       <c r="R40" s="29"/>
       <c r="S40" s="21">
         <f>SUM(S3:S39)</f>
-        <v>155.01500000000001</v>
+        <v>130.626</v>
       </c>
       <c r="T40" s="25"/>
       <c r="U40" s="3"/>
@@ -4505,24 +4508,24 @@
       <c r="I41" s="25"/>
       <c r="J41" s="27"/>
       <c r="K41" s="25"/>
-      <c r="L41" s="112" t="s">
+      <c r="L41" s="132" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="112"/>
-      <c r="N41" s="112"/>
-      <c r="O41" s="112"/>
+      <c r="M41" s="132"/>
+      <c r="N41" s="132"/>
+      <c r="O41" s="132"/>
       <c r="P41" s="21">
         <f>SUM(P3:P39)</f>
-        <v>31.980499999999996</v>
+        <v>26.651699999999995</v>
       </c>
       <c r="Q41" s="21">
         <f>Q40/5</f>
-        <v>40.003740000000001</v>
+        <v>33.609179999999995</v>
       </c>
       <c r="R41" s="26"/>
       <c r="S41" s="28">
         <f>S40/5</f>
-        <v>31.003000000000004</v>
+        <v>26.1252</v>
       </c>
       <c r="T41" s="25"/>
       <c r="U41" s="3"/>
@@ -4794,12 +4797,12 @@
     <hyperlink ref="N23" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
     <hyperlink ref="N24" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
     <hyperlink ref="N25" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N26" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N26" r:id="rId20" display="LCSC" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
     <hyperlink ref="N27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
     <hyperlink ref="N28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
     <hyperlink ref="N29" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
     <hyperlink ref="N30" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="N31" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N31" r:id="rId25" display="LCSC" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
     <hyperlink ref="N32" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
     <hyperlink ref="N33" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
     <hyperlink ref="N34" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>

</xml_diff>